<commit_message>
Add Brand entity with config, mapping, and seeding
Introduced the Brand entity to the domain model, including its configuration, mapping, data record, and seeder. Updated DbContext to support Brands. Increased Category description length to 1000. Changed CategoryRecord and BranchRecord to internal. Updated DatabaseSeeder and Excel data to support Brands.
</commit_message>
<xml_diff>
--- a/src/External/ConvenienceStore.Persistence/Data/ConvenienceStoreData.xlsx
+++ b/src/External/ConvenienceStore.Persistence/Data/ConvenienceStoreData.xlsx
@@ -1,14 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30318"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30305"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="12" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B62D74E2-CB2C-4E0F-BCC6-A9AC9175A74F}"/>
+  <xr:revisionPtr revIDLastSave="26" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{25FF3874-0683-4381-AF56-0F4E3557A6E7}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Categories" sheetId="1" r:id="rId1"/>
+    <sheet name="Brands" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="103">
   <si>
     <t>Id</t>
   </si>
@@ -189,6 +190,186 @@
   </si>
   <si>
     <t>Limited-time products, holiday items, gift sets, and promotional merchandise.</t>
+  </si>
+  <si>
+    <t>Vinamilk</t>
+  </si>
+  <si>
+    <t>Thương hiệu sữa và các sản phẩm từ sữa hàng đầu Việt Nam với đa dạng sữa tươi, sữa chua và đồ uống dinh dưỡng.</t>
+  </si>
+  <si>
+    <t>TH true MILK</t>
+  </si>
+  <si>
+    <t>Thương hiệu sữa nổi tiếng với các sản phẩm sữa tươi, sữa hạt và đồ uống từ nguyên liệu tự nhiên.</t>
+  </si>
+  <si>
+    <t>Milo</t>
+  </si>
+  <si>
+    <t>Thương hiệu thức uống lúa mạch và ca cao nổi tiếng, cung cấp năng lượng cho trẻ em và người năng động.</t>
+  </si>
+  <si>
+    <t>Coca-Cola</t>
+  </si>
+  <si>
+    <t>Thương hiệu nước giải khát toàn cầu với các sản phẩm nước ngọt có ga, nước trái cây và trà.</t>
+  </si>
+  <si>
+    <t>Pepsi</t>
+  </si>
+  <si>
+    <t>Thương hiệu nước giải khát nổi tiếng với nhiều dòng nước có ga, trà và nước tăng lực.</t>
+  </si>
+  <si>
+    <t>Sting</t>
+  </si>
+  <si>
+    <t>Thương hiệu nước tăng lực phổ biến với nhiều hương vị trái cây.</t>
+  </si>
+  <si>
+    <t>Red Bull</t>
+  </si>
+  <si>
+    <t>Thương hiệu nước tăng lực được phân phối rộng rãi tại Việt Nam.</t>
+  </si>
+  <si>
+    <t>Oishi</t>
+  </si>
+  <si>
+    <t>Thương hiệu bánh snack, khoai tây chiên và bánh kẹo được ưa chuộng tại châu Á.</t>
+  </si>
+  <si>
+    <t>Orion</t>
+  </si>
+  <si>
+    <t>Thương hiệu bánh kẹo Hàn Quốc nổi tiếng với ChocoPie, Custas và nhiều loại bánh khác.</t>
+  </si>
+  <si>
+    <t>Kinh Đô</t>
+  </si>
+  <si>
+    <t>Thương hiệu bánh kẹo Việt Nam với đa dạng bánh quy, bánh trung thu và bánh snack.</t>
+  </si>
+  <si>
+    <t>Acecook</t>
+  </si>
+  <si>
+    <t>Nhà sản xuất mì ăn liền hàng đầu Việt Nam với các dòng Hảo Hảo, Modern và Đệ Nhất.</t>
+  </si>
+  <si>
+    <t>Omachi</t>
+  </si>
+  <si>
+    <t>Thương hiệu mì ăn liền cao cấp làm từ khoai tây của Masan Consumer.</t>
+  </si>
+  <si>
+    <t>Kokomi</t>
+  </si>
+  <si>
+    <t>Thương hiệu mì ăn liền phổ thông với nhiều hương vị phù hợp khẩu vị Việt Nam.</t>
+  </si>
+  <si>
+    <t>Vifon</t>
+  </si>
+  <si>
+    <t>Thương hiệu mì, phở, bún ăn liền lâu đời của Việt Nam.</t>
+  </si>
+  <si>
+    <t>Lay's</t>
+  </si>
+  <si>
+    <t>Thương hiệu khoai tây chiên nổi tiếng với nhiều hương vị đa dạng.</t>
+  </si>
+  <si>
+    <t>Pringles</t>
+  </si>
+  <si>
+    <t>Thương hiệu snack khoai tây dạng lon với thiết kế đặc trưng và nhiều hương vị.</t>
+  </si>
+  <si>
+    <t>Poca</t>
+  </si>
+  <si>
+    <t>Thương hiệu snack khoai tây của PepsiCo, sản xuất tại Việt Nam.</t>
+  </si>
+  <si>
+    <t>Nescafé</t>
+  </si>
+  <si>
+    <t>Thương hiệu cà phê hòa tan nổi tiếng của Nestlé.</t>
+  </si>
+  <si>
+    <t>G7</t>
+  </si>
+  <si>
+    <t>Thương hiệu cà phê hòa tan của Trung Nguyên Legend.</t>
+  </si>
+  <si>
+    <t>Highlands Coffee</t>
+  </si>
+  <si>
+    <t>Thương hiệu cà phê Việt Nam có các sản phẩm cà phê đóng lon và đóng chai.</t>
+  </si>
+  <si>
+    <t>C2</t>
+  </si>
+  <si>
+    <t>Thương hiệu trà xanh đóng chai phổ biến với nhiều hương vị.</t>
+  </si>
+  <si>
+    <t>Wonderfarm</t>
+  </si>
+  <si>
+    <t>Thương hiệu đồ uống đóng hộp như trà, nước trái cây và nước yến.</t>
+  </si>
+  <si>
+    <t>Number One</t>
+  </si>
+  <si>
+    <t>Thương hiệu nước tăng lực và nước giải khát của Tân Hiệp Phát.</t>
+  </si>
+  <si>
+    <t>Aquafina</t>
+  </si>
+  <si>
+    <t>Thương hiệu nước uống tinh khiết đóng chai của PepsiCo.</t>
+  </si>
+  <si>
+    <t>Lavie</t>
+  </si>
+  <si>
+    <t>Thương hiệu nước khoáng thiên nhiên đóng chai phổ biến tại Việt Nam.</t>
+  </si>
+  <si>
+    <t>Hảo Hảo</t>
+  </si>
+  <si>
+    <t>Thương hiệu mì ăn liền nổi tiếng nhất của Acecook, thường được quản lý như một brand riêng trong bán lẻ.</t>
+  </si>
+  <si>
+    <t>ChocoPie</t>
+  </si>
+  <si>
+    <t>Thương hiệu bánh mềm phủ socola nổi tiếng của Orion.</t>
+  </si>
+  <si>
+    <t>KitKat</t>
+  </si>
+  <si>
+    <t>Thương hiệu bánh xốp phủ socola nổi tiếng của Nestlé.</t>
+  </si>
+  <si>
+    <t>Mentos</t>
+  </si>
+  <si>
+    <t>Thương hiệu kẹo bạc hà và kẹo dẻo được bán phổ biến tại cửa hàng tiện lợi.</t>
+  </si>
+  <si>
+    <t>Alpenliebe</t>
+  </si>
+  <si>
+    <t>Thương hiệu kẹo sữa và caramel được ưa chuộng tại Việt Nam.</t>
   </si>
 </sst>
 </file>
@@ -788,4 +969,355 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{748F4E0F-BC34-4228-867E-9D0F821705DC}">
+  <dimension ref="A1:C31"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C5" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>53</v>
+      </c>
+      <c r="C7" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>55</v>
+      </c>
+      <c r="C8" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>57</v>
+      </c>
+      <c r="C9" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>59</v>
+      </c>
+      <c r="C10" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C11" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>63</v>
+      </c>
+      <c r="C12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>65</v>
+      </c>
+      <c r="C13" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>67</v>
+      </c>
+      <c r="C14" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>69</v>
+      </c>
+      <c r="C15" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>71</v>
+      </c>
+      <c r="C16" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>73</v>
+      </c>
+      <c r="C17" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>75</v>
+      </c>
+      <c r="C18" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>77</v>
+      </c>
+      <c r="C19" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>79</v>
+      </c>
+      <c r="C20" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>81</v>
+      </c>
+      <c r="C21" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>83</v>
+      </c>
+      <c r="C22" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
+        <v>85</v>
+      </c>
+      <c r="C23" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="s">
+        <v>87</v>
+      </c>
+      <c r="C24" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>89</v>
+      </c>
+      <c r="C25" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>91</v>
+      </c>
+      <c r="C26" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>93</v>
+      </c>
+      <c r="C27" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
+        <v>95</v>
+      </c>
+      <c r="C28" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="s">
+        <v>97</v>
+      </c>
+      <c r="C29" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="s">
+        <v>99</v>
+      </c>
+      <c r="C30" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="s">
+        <v>101</v>
+      </c>
+      <c r="C31" t="s">
+        <v>102</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add CQRS query, DTO, and repo/service for products
Implemented GetAllProductQuery and specification for product retrieval using CQRS. Added ProductResponse DTO, IProductService interface with stub, and IProductRespository with implementation. Introduced AutoMapper profile for Product mapping. Updated Excel data file.
</commit_message>
<xml_diff>
--- a/src/External/ConvenienceStore.Persistence/Data/ConvenienceStoreData.xlsx
+++ b/src/External/ConvenienceStore.Persistence/Data/ConvenienceStoreData.xlsx
@@ -1,15 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30305"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30318"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="26" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{25FF3874-0683-4381-AF56-0F4E3557A6E7}"/>
+  <xr:revisionPtr revIDLastSave="50" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0002D883-D255-43C5-BD49-3325098AB764}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Categories" sheetId="1" r:id="rId1"/>
     <sheet name="Brands" sheetId="2" r:id="rId2"/>
+    <sheet name="Products" sheetId="3" r:id="rId3"/>
+    <sheet name="ProductStocks" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -35,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="302">
   <si>
     <t>Id</t>
   </si>
@@ -370,6 +372,603 @@
   </si>
   <si>
     <t>Thương hiệu kẹo sữa và caramel được ưa chuộng tại Việt Nam.</t>
+  </si>
+  <si>
+    <t>CategoryId</t>
+  </si>
+  <si>
+    <t>BrandId</t>
+  </si>
+  <si>
+    <t>TH True Milk Fresh Milk 180ml</t>
+  </si>
+  <si>
+    <t>Fresh milk 180ml</t>
+  </si>
+  <si>
+    <t>TH True Milk Chocolate Milk 180ml</t>
+  </si>
+  <si>
+    <t>Chocolate milk</t>
+  </si>
+  <si>
+    <t>Milo Chocolate Drink 180ml</t>
+  </si>
+  <si>
+    <t>Chocolate malt drink</t>
+  </si>
+  <si>
+    <t>Coca-Cola Original 330ml</t>
+  </si>
+  <si>
+    <t>Soft drink can</t>
+  </si>
+  <si>
+    <t>Coca-Cola Zero 330ml</t>
+  </si>
+  <si>
+    <t>Sugar free cola</t>
+  </si>
+  <si>
+    <t>Pepsi Cola 330ml</t>
+  </si>
+  <si>
+    <t>Cola soft drink</t>
+  </si>
+  <si>
+    <t>Sting Red 330ml</t>
+  </si>
+  <si>
+    <t>Energy drink</t>
+  </si>
+  <si>
+    <t>Red Bull Energy Drink 250ml</t>
+  </si>
+  <si>
+    <t>Oishi Potato Chips Original</t>
+  </si>
+  <si>
+    <t>Potato chips</t>
+  </si>
+  <si>
+    <t>Oishi Prawn Crackers</t>
+  </si>
+  <si>
+    <t>Snack crackers</t>
+  </si>
+  <si>
+    <t>Orion ChocoPie 6P</t>
+  </si>
+  <si>
+    <t>Chocolate pie</t>
+  </si>
+  <si>
+    <t>Orion Custas Cake</t>
+  </si>
+  <si>
+    <t>Custard cake</t>
+  </si>
+  <si>
+    <t>Kin Do Butter Cookies</t>
+  </si>
+  <si>
+    <t>Butter cookies</t>
+  </si>
+  <si>
+    <t>Acecook Hao Hao Shrimp Noodles</t>
+  </si>
+  <si>
+    <t>Instant noodles</t>
+  </si>
+  <si>
+    <t>Omachi Beef Noodles</t>
+  </si>
+  <si>
+    <t>Premium instant noodles</t>
+  </si>
+  <si>
+    <t>Kokomi Chicken Noodles</t>
+  </si>
+  <si>
+    <t>Vifon Pho Bo</t>
+  </si>
+  <si>
+    <t>Instant pho</t>
+  </si>
+  <si>
+    <t>Lay's Classic Chips</t>
+  </si>
+  <si>
+    <t>Lay's BBQ Chips</t>
+  </si>
+  <si>
+    <t>BBQ potato chips</t>
+  </si>
+  <si>
+    <t>Pringles Original</t>
+  </si>
+  <si>
+    <t>Potato crisps</t>
+  </si>
+  <si>
+    <t>Poca Seaweed Chips</t>
+  </si>
+  <si>
+    <t>Seaweed chips</t>
+  </si>
+  <si>
+    <t>Nescafe 3in1 Coffee</t>
+  </si>
+  <si>
+    <t>Coffee mix</t>
+  </si>
+  <si>
+    <t>Highlands Coffee Can</t>
+  </si>
+  <si>
+    <t>Ready coffee</t>
+  </si>
+  <si>
+    <t>C2 Green Tea</t>
+  </si>
+  <si>
+    <t>Tea drink</t>
+  </si>
+  <si>
+    <t>Wonderfarm Grass Jelly</t>
+  </si>
+  <si>
+    <t>Grass jelly drink</t>
+  </si>
+  <si>
+    <t>Number One Energy Drink</t>
+  </si>
+  <si>
+    <t>Aquafina Water 500ml</t>
+  </si>
+  <si>
+    <t>Drinking water</t>
+  </si>
+  <si>
+    <t>LaVie Water 500ml</t>
+  </si>
+  <si>
+    <t>Mineral water</t>
+  </si>
+  <si>
+    <t>Hao Hao Sour Shrimp Noodles</t>
+  </si>
+  <si>
+    <t>Choco Pie Banana</t>
+  </si>
+  <si>
+    <t>Banana pie</t>
+  </si>
+  <si>
+    <t>KitKat 4 Finger</t>
+  </si>
+  <si>
+    <t>Chocolate wafer</t>
+  </si>
+  <si>
+    <t>Mentos Mint</t>
+  </si>
+  <si>
+    <t>Chewy mint candy</t>
+  </si>
+  <si>
+    <t>Alpenliebe Milk Candy</t>
+  </si>
+  <si>
+    <t>Milk candy</t>
+  </si>
+  <si>
+    <t>TH True Yogurt Drink</t>
+  </si>
+  <si>
+    <t>Yogurt drink</t>
+  </si>
+  <si>
+    <t>Milo Active Go</t>
+  </si>
+  <si>
+    <t>Chocolate drink</t>
+  </si>
+  <si>
+    <t>Coca-Cola Vanilla</t>
+  </si>
+  <si>
+    <t>Vanilla cola</t>
+  </si>
+  <si>
+    <t>Pepsi Black</t>
+  </si>
+  <si>
+    <t>Red Bull Sugar Free</t>
+  </si>
+  <si>
+    <t>Oishi Seaweed Snack</t>
+  </si>
+  <si>
+    <t>Seaweed snack</t>
+  </si>
+  <si>
+    <t>Orion Goute Cookies</t>
+  </si>
+  <si>
+    <t>Cookies</t>
+  </si>
+  <si>
+    <t>Acecook Siu Kay Noodles</t>
+  </si>
+  <si>
+    <t>Omachi Kimchi Noodles</t>
+  </si>
+  <si>
+    <t>Kimchi noodles</t>
+  </si>
+  <si>
+    <t>Kokomi Sour Soup Noodles</t>
+  </si>
+  <si>
+    <t>Vifon Instant Pho Chicken</t>
+  </si>
+  <si>
+    <t>Chicken pho</t>
+  </si>
+  <si>
+    <t>Lay's Sour Cream Chips</t>
+  </si>
+  <si>
+    <t>Pringles BBQ</t>
+  </si>
+  <si>
+    <t>Poca Corn Chips</t>
+  </si>
+  <si>
+    <t>Corn snack</t>
+  </si>
+  <si>
+    <t>Nescafe Black Coffee</t>
+  </si>
+  <si>
+    <t>Black coffee</t>
+  </si>
+  <si>
+    <t>Highlands Freeze Coffee</t>
+  </si>
+  <si>
+    <t>Canned coffee</t>
+  </si>
+  <si>
+    <t>C2 Lemon Tea</t>
+  </si>
+  <si>
+    <t>Lemon tea</t>
+  </si>
+  <si>
+    <t>Wonderfarm Soya Milk</t>
+  </si>
+  <si>
+    <t>Soy milk</t>
+  </si>
+  <si>
+    <t>Number One Active</t>
+  </si>
+  <si>
+    <t>Aquafina Sparkling</t>
+  </si>
+  <si>
+    <t>Sparkling water</t>
+  </si>
+  <si>
+    <t>LaVie Sparkling</t>
+  </si>
+  <si>
+    <t>KitKat Dark</t>
+  </si>
+  <si>
+    <t>Dark chocolate wafer</t>
+  </si>
+  <si>
+    <t>Mentos Fruit</t>
+  </si>
+  <si>
+    <t>Fruit candy</t>
+  </si>
+  <si>
+    <t>Alpenliebe Coffee</t>
+  </si>
+  <si>
+    <t>Coffee candy</t>
+  </si>
+  <si>
+    <t>Bread Sandwich</t>
+  </si>
+  <si>
+    <t>Bread sandwich</t>
+  </si>
+  <si>
+    <t>Croissant Butter</t>
+  </si>
+  <si>
+    <t>Butter croissant</t>
+  </si>
+  <si>
+    <t>Mini Pizza</t>
+  </si>
+  <si>
+    <t>Ready pizza</t>
+  </si>
+  <si>
+    <t>Fried Chicken Rice</t>
+  </si>
+  <si>
+    <t>Microwave meal</t>
+  </si>
+  <si>
+    <t>Pork Fried Rice</t>
+  </si>
+  <si>
+    <t>Ready meal</t>
+  </si>
+  <si>
+    <t>Chicken Sausage</t>
+  </si>
+  <si>
+    <t>Sausage</t>
+  </si>
+  <si>
+    <t>Fish Ball</t>
+  </si>
+  <si>
+    <t>Frozen fish ball</t>
+  </si>
+  <si>
+    <t>Ice Cream Vanilla</t>
+  </si>
+  <si>
+    <t>Vanilla ice cream</t>
+  </si>
+  <si>
+    <t>Ice Cream Chocolate</t>
+  </si>
+  <si>
+    <t>Chocolate ice cream</t>
+  </si>
+  <si>
+    <t>Fresh Apple</t>
+  </si>
+  <si>
+    <t>Fresh apple</t>
+  </si>
+  <si>
+    <t>Fresh Banana</t>
+  </si>
+  <si>
+    <t>Banana</t>
+  </si>
+  <si>
+    <t>Fresh Orange</t>
+  </si>
+  <si>
+    <t>Orange</t>
+  </si>
+  <si>
+    <t>Fresh Lettuce</t>
+  </si>
+  <si>
+    <t>Lettuce</t>
+  </si>
+  <si>
+    <t>Chicken Breast</t>
+  </si>
+  <si>
+    <t>Fresh chicken</t>
+  </si>
+  <si>
+    <t>Pork Slice</t>
+  </si>
+  <si>
+    <t>Fresh pork</t>
+  </si>
+  <si>
+    <t>Eggs 10 Pack</t>
+  </si>
+  <si>
+    <t>Chicken eggs</t>
+  </si>
+  <si>
+    <t>Fresh Milk Bread</t>
+  </si>
+  <si>
+    <t>Milk bread</t>
+  </si>
+  <si>
+    <t>Chocolate Donut</t>
+  </si>
+  <si>
+    <t>Donut</t>
+  </si>
+  <si>
+    <t>Cheese Cake Slice</t>
+  </si>
+  <si>
+    <t>Cake slice</t>
+  </si>
+  <si>
+    <t>Instant Rice Bowl</t>
+  </si>
+  <si>
+    <t>Instant rice</t>
+  </si>
+  <si>
+    <t>Cup Noodles Seafood</t>
+  </si>
+  <si>
+    <t>Cup noodles</t>
+  </si>
+  <si>
+    <t>Cup Noodles Beef</t>
+  </si>
+  <si>
+    <t>Canned Tuna</t>
+  </si>
+  <si>
+    <t>Tuna can</t>
+  </si>
+  <si>
+    <t>Canned Sardines</t>
+  </si>
+  <si>
+    <t>Sardines can</t>
+  </si>
+  <si>
+    <t>Baked Beans</t>
+  </si>
+  <si>
+    <t>Baked beans</t>
+  </si>
+  <si>
+    <t>Tomato Ketchup</t>
+  </si>
+  <si>
+    <t>Ketchup bottle</t>
+  </si>
+  <si>
+    <t>Mayonnaise</t>
+  </si>
+  <si>
+    <t>Shampoo 170ml</t>
+  </si>
+  <si>
+    <t>Hair shampoo</t>
+  </si>
+  <si>
+    <t>Body Wash 250ml</t>
+  </si>
+  <si>
+    <t>Body wash</t>
+  </si>
+  <si>
+    <t>Toothpaste 150g</t>
+  </si>
+  <si>
+    <t>Toothpaste</t>
+  </si>
+  <si>
+    <t>Laundry Detergent</t>
+  </si>
+  <si>
+    <t>Liquid detergent</t>
+  </si>
+  <si>
+    <t>Dishwashing Liquid</t>
+  </si>
+  <si>
+    <t>Dish soap</t>
+  </si>
+  <si>
+    <t>Tissue Box</t>
+  </si>
+  <si>
+    <t>Tissue paper</t>
+  </si>
+  <si>
+    <t>Cat Food 500g</t>
+  </si>
+  <si>
+    <t>Cat food</t>
+  </si>
+  <si>
+    <t>Dog Food 1kg</t>
+  </si>
+  <si>
+    <t>Dog food</t>
+  </si>
+  <si>
+    <t>Baby Diapers M</t>
+  </si>
+  <si>
+    <t>Diapers</t>
+  </si>
+  <si>
+    <t>Baby Wipes</t>
+  </si>
+  <si>
+    <t>Wet wipes</t>
+  </si>
+  <si>
+    <t>Cigarette Pack A</t>
+  </si>
+  <si>
+    <t>Cigarettes</t>
+  </si>
+  <si>
+    <t>Cigarette Pack B</t>
+  </si>
+  <si>
+    <t>Beer Can 330ml</t>
+  </si>
+  <si>
+    <t>Beer can</t>
+  </si>
+  <si>
+    <t>Beer Bottle 500ml</t>
+  </si>
+  <si>
+    <t>Beer bottle</t>
+  </si>
+  <si>
+    <t>Moon Cake</t>
+  </si>
+  <si>
+    <t>Seasonal cake</t>
+  </si>
+  <si>
+    <t>Gift Snack Box</t>
+  </si>
+  <si>
+    <t>Gift combo</t>
+  </si>
+  <si>
+    <t>UnitPrice</t>
+  </si>
+  <si>
+    <t>Unit</t>
+  </si>
+  <si>
+    <t>QuantityOnHand</t>
+  </si>
+  <si>
+    <t>ProductId</t>
+  </si>
+  <si>
+    <t>Bottle</t>
+  </si>
+  <si>
+    <t>Box</t>
+  </si>
+  <si>
+    <t>Can</t>
+  </si>
+  <si>
+    <t>Bag</t>
+  </si>
+  <si>
+    <t>Pack</t>
+  </si>
+  <si>
+    <t>Piece</t>
+  </si>
+  <si>
+    <t>Tub</t>
+  </si>
+  <si>
+    <t>Kg</t>
+  </si>
+  <si>
+    <t>Cup</t>
   </si>
 </sst>
 </file>
@@ -1320,4 +1919,3465 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01D486D1-C735-4FA3-BB9F-F95DF0BBE0F4}">
+  <dimension ref="A1:E101"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="3" max="3" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>103</v>
+      </c>
+      <c r="E1" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C2" t="s">
+        <v>106</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>107</v>
+      </c>
+      <c r="C3" t="s">
+        <v>108</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>109</v>
+      </c>
+      <c r="C4" t="s">
+        <v>110</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>111</v>
+      </c>
+      <c r="C5" t="s">
+        <v>112</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>113</v>
+      </c>
+      <c r="C6" t="s">
+        <v>114</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>115</v>
+      </c>
+      <c r="C7" t="s">
+        <v>116</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>117</v>
+      </c>
+      <c r="C8" t="s">
+        <v>118</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>119</v>
+      </c>
+      <c r="C9" t="s">
+        <v>118</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>120</v>
+      </c>
+      <c r="C10" t="s">
+        <v>121</v>
+      </c>
+      <c r="D10">
+        <v>2</v>
+      </c>
+      <c r="E10">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>122</v>
+      </c>
+      <c r="C11" t="s">
+        <v>123</v>
+      </c>
+      <c r="D11">
+        <v>2</v>
+      </c>
+      <c r="E11">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>124</v>
+      </c>
+      <c r="C12" t="s">
+        <v>125</v>
+      </c>
+      <c r="D12">
+        <v>10</v>
+      </c>
+      <c r="E12">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>126</v>
+      </c>
+      <c r="C13" t="s">
+        <v>127</v>
+      </c>
+      <c r="D13">
+        <v>5</v>
+      </c>
+      <c r="E13">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>128</v>
+      </c>
+      <c r="C14" t="s">
+        <v>129</v>
+      </c>
+      <c r="D14">
+        <v>10</v>
+      </c>
+      <c r="E14">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>130</v>
+      </c>
+      <c r="C15" t="s">
+        <v>131</v>
+      </c>
+      <c r="D15">
+        <v>3</v>
+      </c>
+      <c r="E15">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>132</v>
+      </c>
+      <c r="C16" t="s">
+        <v>133</v>
+      </c>
+      <c r="D16">
+        <v>3</v>
+      </c>
+      <c r="E16">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>134</v>
+      </c>
+      <c r="C17" t="s">
+        <v>131</v>
+      </c>
+      <c r="D17">
+        <v>3</v>
+      </c>
+      <c r="E17">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>135</v>
+      </c>
+      <c r="C18" t="s">
+        <v>136</v>
+      </c>
+      <c r="D18">
+        <v>3</v>
+      </c>
+      <c r="E18">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>137</v>
+      </c>
+      <c r="C19" t="s">
+        <v>121</v>
+      </c>
+      <c r="D19">
+        <v>2</v>
+      </c>
+      <c r="E19">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>138</v>
+      </c>
+      <c r="C20" t="s">
+        <v>139</v>
+      </c>
+      <c r="D20">
+        <v>2</v>
+      </c>
+      <c r="E20">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>140</v>
+      </c>
+      <c r="C21" t="s">
+        <v>141</v>
+      </c>
+      <c r="D21">
+        <v>2</v>
+      </c>
+      <c r="E21">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>142</v>
+      </c>
+      <c r="C22" t="s">
+        <v>143</v>
+      </c>
+      <c r="D22">
+        <v>2</v>
+      </c>
+      <c r="E22">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
+        <v>144</v>
+      </c>
+      <c r="C23" t="s">
+        <v>145</v>
+      </c>
+      <c r="D23">
+        <v>1</v>
+      </c>
+      <c r="E23">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="s">
+        <v>146</v>
+      </c>
+      <c r="C24" t="s">
+        <v>147</v>
+      </c>
+      <c r="D24">
+        <v>1</v>
+      </c>
+      <c r="E24">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>148</v>
+      </c>
+      <c r="C25" t="s">
+        <v>149</v>
+      </c>
+      <c r="D25">
+        <v>1</v>
+      </c>
+      <c r="E25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>150</v>
+      </c>
+      <c r="C26" t="s">
+        <v>151</v>
+      </c>
+      <c r="D26">
+        <v>1</v>
+      </c>
+      <c r="E26">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>152</v>
+      </c>
+      <c r="C27" t="s">
+        <v>118</v>
+      </c>
+      <c r="D27">
+        <v>1</v>
+      </c>
+      <c r="E27">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
+        <v>153</v>
+      </c>
+      <c r="C28" t="s">
+        <v>154</v>
+      </c>
+      <c r="D28">
+        <v>1</v>
+      </c>
+      <c r="E28">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="s">
+        <v>155</v>
+      </c>
+      <c r="C29" t="s">
+        <v>156</v>
+      </c>
+      <c r="D29">
+        <v>1</v>
+      </c>
+      <c r="E29">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="s">
+        <v>157</v>
+      </c>
+      <c r="C30" t="s">
+        <v>131</v>
+      </c>
+      <c r="D30">
+        <v>3</v>
+      </c>
+      <c r="E30">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="s">
+        <v>158</v>
+      </c>
+      <c r="C31" t="s">
+        <v>159</v>
+      </c>
+      <c r="D31">
+        <v>10</v>
+      </c>
+      <c r="E31">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="s">
+        <v>160</v>
+      </c>
+      <c r="C32" t="s">
+        <v>161</v>
+      </c>
+      <c r="D32">
+        <v>10</v>
+      </c>
+      <c r="E32">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" t="s">
+        <v>162</v>
+      </c>
+      <c r="C33" t="s">
+        <v>163</v>
+      </c>
+      <c r="D33">
+        <v>10</v>
+      </c>
+      <c r="E33">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" t="s">
+        <v>164</v>
+      </c>
+      <c r="C34" t="s">
+        <v>165</v>
+      </c>
+      <c r="D34">
+        <v>10</v>
+      </c>
+      <c r="E34">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" t="s">
+        <v>166</v>
+      </c>
+      <c r="C35" t="s">
+        <v>167</v>
+      </c>
+      <c r="D35">
+        <v>1</v>
+      </c>
+      <c r="E35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36" t="s">
+        <v>168</v>
+      </c>
+      <c r="C36" t="s">
+        <v>169</v>
+      </c>
+      <c r="D36">
+        <v>1</v>
+      </c>
+      <c r="E36">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37" t="s">
+        <v>170</v>
+      </c>
+      <c r="C37" t="s">
+        <v>171</v>
+      </c>
+      <c r="D37">
+        <v>1</v>
+      </c>
+      <c r="E37">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38" t="s">
+        <v>172</v>
+      </c>
+      <c r="C38" t="s">
+        <v>114</v>
+      </c>
+      <c r="D38">
+        <v>1</v>
+      </c>
+      <c r="E38">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5">
+      <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39" t="s">
+        <v>173</v>
+      </c>
+      <c r="C39" t="s">
+        <v>118</v>
+      </c>
+      <c r="D39">
+        <v>1</v>
+      </c>
+      <c r="E39">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40" t="s">
+        <v>174</v>
+      </c>
+      <c r="C40" t="s">
+        <v>175</v>
+      </c>
+      <c r="D40">
+        <v>2</v>
+      </c>
+      <c r="E40">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41" t="s">
+        <v>176</v>
+      </c>
+      <c r="C41" t="s">
+        <v>177</v>
+      </c>
+      <c r="D41">
+        <v>10</v>
+      </c>
+      <c r="E41">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5">
+      <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42" t="s">
+        <v>178</v>
+      </c>
+      <c r="C42" t="s">
+        <v>131</v>
+      </c>
+      <c r="D42">
+        <v>3</v>
+      </c>
+      <c r="E42">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43" t="s">
+        <v>179</v>
+      </c>
+      <c r="C43" t="s">
+        <v>180</v>
+      </c>
+      <c r="D43">
+        <v>3</v>
+      </c>
+      <c r="E43">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5">
+      <c r="A44">
+        <v>43</v>
+      </c>
+      <c r="B44" t="s">
+        <v>181</v>
+      </c>
+      <c r="C44" t="s">
+        <v>131</v>
+      </c>
+      <c r="D44">
+        <v>3</v>
+      </c>
+      <c r="E44">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5">
+      <c r="A45">
+        <v>44</v>
+      </c>
+      <c r="B45" t="s">
+        <v>182</v>
+      </c>
+      <c r="C45" t="s">
+        <v>183</v>
+      </c>
+      <c r="D45">
+        <v>3</v>
+      </c>
+      <c r="E45">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5">
+      <c r="A46">
+        <v>45</v>
+      </c>
+      <c r="B46" t="s">
+        <v>184</v>
+      </c>
+      <c r="C46" t="s">
+        <v>121</v>
+      </c>
+      <c r="D46">
+        <v>2</v>
+      </c>
+      <c r="E46">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5">
+      <c r="A47">
+        <v>46</v>
+      </c>
+      <c r="B47" t="s">
+        <v>185</v>
+      </c>
+      <c r="C47" t="s">
+        <v>141</v>
+      </c>
+      <c r="D47">
+        <v>2</v>
+      </c>
+      <c r="E47">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5">
+      <c r="A48">
+        <v>47</v>
+      </c>
+      <c r="B48" t="s">
+        <v>186</v>
+      </c>
+      <c r="C48" t="s">
+        <v>187</v>
+      </c>
+      <c r="D48">
+        <v>2</v>
+      </c>
+      <c r="E48">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5">
+      <c r="A49">
+        <v>48</v>
+      </c>
+      <c r="B49" t="s">
+        <v>188</v>
+      </c>
+      <c r="C49" t="s">
+        <v>189</v>
+      </c>
+      <c r="D49">
+        <v>1</v>
+      </c>
+      <c r="E49">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5">
+      <c r="A50">
+        <v>49</v>
+      </c>
+      <c r="B50" t="s">
+        <v>190</v>
+      </c>
+      <c r="C50" t="s">
+        <v>191</v>
+      </c>
+      <c r="D50">
+        <v>1</v>
+      </c>
+      <c r="E50">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5">
+      <c r="A51">
+        <v>50</v>
+      </c>
+      <c r="B51" t="s">
+        <v>192</v>
+      </c>
+      <c r="C51" t="s">
+        <v>193</v>
+      </c>
+      <c r="D51">
+        <v>1</v>
+      </c>
+      <c r="E51">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5">
+      <c r="A52">
+        <v>51</v>
+      </c>
+      <c r="B52" t="s">
+        <v>194</v>
+      </c>
+      <c r="C52" t="s">
+        <v>195</v>
+      </c>
+      <c r="D52">
+        <v>1</v>
+      </c>
+      <c r="E52">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5">
+      <c r="A53">
+        <v>52</v>
+      </c>
+      <c r="B53" t="s">
+        <v>196</v>
+      </c>
+      <c r="C53" t="s">
+        <v>118</v>
+      </c>
+      <c r="D53">
+        <v>1</v>
+      </c>
+      <c r="E53">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5">
+      <c r="A54">
+        <v>53</v>
+      </c>
+      <c r="B54" t="s">
+        <v>197</v>
+      </c>
+      <c r="C54" t="s">
+        <v>198</v>
+      </c>
+      <c r="D54">
+        <v>1</v>
+      </c>
+      <c r="E54">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5">
+      <c r="A55">
+        <v>54</v>
+      </c>
+      <c r="B55" t="s">
+        <v>199</v>
+      </c>
+      <c r="C55" t="s">
+        <v>198</v>
+      </c>
+      <c r="D55">
+        <v>1</v>
+      </c>
+      <c r="E55">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5">
+      <c r="A56">
+        <v>55</v>
+      </c>
+      <c r="B56" t="s">
+        <v>200</v>
+      </c>
+      <c r="C56" t="s">
+        <v>201</v>
+      </c>
+      <c r="D56">
+        <v>10</v>
+      </c>
+      <c r="E56">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5">
+      <c r="A57">
+        <v>56</v>
+      </c>
+      <c r="B57" t="s">
+        <v>202</v>
+      </c>
+      <c r="C57" t="s">
+        <v>203</v>
+      </c>
+      <c r="D57">
+        <v>10</v>
+      </c>
+      <c r="E57">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5">
+      <c r="A58">
+        <v>57</v>
+      </c>
+      <c r="B58" t="s">
+        <v>204</v>
+      </c>
+      <c r="C58" t="s">
+        <v>205</v>
+      </c>
+      <c r="D58">
+        <v>10</v>
+      </c>
+      <c r="E58">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5">
+      <c r="A59">
+        <v>58</v>
+      </c>
+      <c r="B59" t="s">
+        <v>206</v>
+      </c>
+      <c r="C59" t="s">
+        <v>207</v>
+      </c>
+      <c r="D59">
+        <v>5</v>
+      </c>
+      <c r="E59">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5">
+      <c r="A60">
+        <v>59</v>
+      </c>
+      <c r="B60" t="s">
+        <v>208</v>
+      </c>
+      <c r="C60" t="s">
+        <v>209</v>
+      </c>
+      <c r="D60">
+        <v>5</v>
+      </c>
+      <c r="E60">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5">
+      <c r="A61">
+        <v>60</v>
+      </c>
+      <c r="B61" t="s">
+        <v>210</v>
+      </c>
+      <c r="C61" t="s">
+        <v>211</v>
+      </c>
+      <c r="D61">
+        <v>17</v>
+      </c>
+      <c r="E61">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5">
+      <c r="A62">
+        <v>61</v>
+      </c>
+      <c r="B62" t="s">
+        <v>212</v>
+      </c>
+      <c r="C62" t="s">
+        <v>213</v>
+      </c>
+      <c r="D62">
+        <v>17</v>
+      </c>
+      <c r="E62">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5">
+      <c r="A63">
+        <v>62</v>
+      </c>
+      <c r="B63" t="s">
+        <v>214</v>
+      </c>
+      <c r="C63" t="s">
+        <v>215</v>
+      </c>
+      <c r="D63">
+        <v>17</v>
+      </c>
+      <c r="E63">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5">
+      <c r="A64">
+        <v>63</v>
+      </c>
+      <c r="B64" t="s">
+        <v>216</v>
+      </c>
+      <c r="C64" t="s">
+        <v>217</v>
+      </c>
+      <c r="D64">
+        <v>8</v>
+      </c>
+      <c r="E64">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5">
+      <c r="A65">
+        <v>64</v>
+      </c>
+      <c r="B65" t="s">
+        <v>218</v>
+      </c>
+      <c r="C65" t="s">
+        <v>219</v>
+      </c>
+      <c r="D65">
+        <v>6</v>
+      </c>
+      <c r="E65">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5">
+      <c r="A66">
+        <v>65</v>
+      </c>
+      <c r="B66" t="s">
+        <v>220</v>
+      </c>
+      <c r="C66" t="s">
+        <v>221</v>
+      </c>
+      <c r="D66">
+        <v>19</v>
+      </c>
+      <c r="E66">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5">
+      <c r="A67">
+        <v>66</v>
+      </c>
+      <c r="B67" t="s">
+        <v>222</v>
+      </c>
+      <c r="C67" t="s">
+        <v>223</v>
+      </c>
+      <c r="D67">
+        <v>19</v>
+      </c>
+      <c r="E67">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5">
+      <c r="A68">
+        <v>67</v>
+      </c>
+      <c r="B68" t="s">
+        <v>224</v>
+      </c>
+      <c r="C68" t="s">
+        <v>225</v>
+      </c>
+      <c r="D68">
+        <v>7</v>
+      </c>
+      <c r="E68">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5">
+      <c r="A69">
+        <v>68</v>
+      </c>
+      <c r="B69" t="s">
+        <v>226</v>
+      </c>
+      <c r="C69" t="s">
+        <v>227</v>
+      </c>
+      <c r="D69">
+        <v>7</v>
+      </c>
+      <c r="E69">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5">
+      <c r="A70">
+        <v>69</v>
+      </c>
+      <c r="B70" t="s">
+        <v>228</v>
+      </c>
+      <c r="C70" t="s">
+        <v>229</v>
+      </c>
+      <c r="D70">
+        <v>7</v>
+      </c>
+      <c r="E70">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5">
+      <c r="A71">
+        <v>70</v>
+      </c>
+      <c r="B71" t="s">
+        <v>230</v>
+      </c>
+      <c r="C71" t="s">
+        <v>231</v>
+      </c>
+      <c r="D71">
+        <v>7</v>
+      </c>
+      <c r="E71">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5">
+      <c r="A72">
+        <v>71</v>
+      </c>
+      <c r="B72" t="s">
+        <v>232</v>
+      </c>
+      <c r="C72" t="s">
+        <v>233</v>
+      </c>
+      <c r="D72">
+        <v>8</v>
+      </c>
+      <c r="E72">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5">
+      <c r="A73">
+        <v>72</v>
+      </c>
+      <c r="B73" t="s">
+        <v>234</v>
+      </c>
+      <c r="C73" t="s">
+        <v>235</v>
+      </c>
+      <c r="D73">
+        <v>8</v>
+      </c>
+      <c r="E73">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5">
+      <c r="A74">
+        <v>73</v>
+      </c>
+      <c r="B74" t="s">
+        <v>236</v>
+      </c>
+      <c r="C74" t="s">
+        <v>237</v>
+      </c>
+      <c r="D74">
+        <v>4</v>
+      </c>
+      <c r="E74">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5">
+      <c r="A75">
+        <v>74</v>
+      </c>
+      <c r="B75" t="s">
+        <v>238</v>
+      </c>
+      <c r="C75" t="s">
+        <v>239</v>
+      </c>
+      <c r="D75">
+        <v>5</v>
+      </c>
+      <c r="E75">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5">
+      <c r="A76">
+        <v>75</v>
+      </c>
+      <c r="B76" t="s">
+        <v>240</v>
+      </c>
+      <c r="C76" t="s">
+        <v>241</v>
+      </c>
+      <c r="D76">
+        <v>5</v>
+      </c>
+      <c r="E76">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5">
+      <c r="A77">
+        <v>76</v>
+      </c>
+      <c r="B77" t="s">
+        <v>242</v>
+      </c>
+      <c r="C77" t="s">
+        <v>243</v>
+      </c>
+      <c r="D77">
+        <v>5</v>
+      </c>
+      <c r="E77">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5">
+      <c r="A78">
+        <v>77</v>
+      </c>
+      <c r="B78" t="s">
+        <v>244</v>
+      </c>
+      <c r="C78" t="s">
+        <v>245</v>
+      </c>
+      <c r="D78">
+        <v>3</v>
+      </c>
+      <c r="E78">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5">
+      <c r="A79">
+        <v>78</v>
+      </c>
+      <c r="B79" t="s">
+        <v>246</v>
+      </c>
+      <c r="C79" t="s">
+        <v>247</v>
+      </c>
+      <c r="D79">
+        <v>3</v>
+      </c>
+      <c r="E79">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5">
+      <c r="A80">
+        <v>79</v>
+      </c>
+      <c r="B80" t="s">
+        <v>248</v>
+      </c>
+      <c r="C80" t="s">
+        <v>247</v>
+      </c>
+      <c r="D80">
+        <v>3</v>
+      </c>
+      <c r="E80">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5">
+      <c r="A81">
+        <v>80</v>
+      </c>
+      <c r="B81" t="s">
+        <v>249</v>
+      </c>
+      <c r="C81" t="s">
+        <v>250</v>
+      </c>
+      <c r="D81">
+        <v>9</v>
+      </c>
+      <c r="E81">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5">
+      <c r="A82">
+        <v>81</v>
+      </c>
+      <c r="B82" t="s">
+        <v>251</v>
+      </c>
+      <c r="C82" t="s">
+        <v>252</v>
+      </c>
+      <c r="D82">
+        <v>9</v>
+      </c>
+      <c r="E82">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5">
+      <c r="A83">
+        <v>82</v>
+      </c>
+      <c r="B83" t="s">
+        <v>253</v>
+      </c>
+      <c r="C83" t="s">
+        <v>254</v>
+      </c>
+      <c r="D83">
+        <v>9</v>
+      </c>
+      <c r="E83">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5">
+      <c r="A84">
+        <v>83</v>
+      </c>
+      <c r="B84" t="s">
+        <v>255</v>
+      </c>
+      <c r="C84" t="s">
+        <v>256</v>
+      </c>
+      <c r="D84">
+        <v>9</v>
+      </c>
+      <c r="E84">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5">
+      <c r="A85">
+        <v>84</v>
+      </c>
+      <c r="B85" t="s">
+        <v>257</v>
+      </c>
+      <c r="C85" t="s">
+        <v>257</v>
+      </c>
+      <c r="D85">
+        <v>9</v>
+      </c>
+      <c r="E85">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5">
+      <c r="A86">
+        <v>85</v>
+      </c>
+      <c r="B86" t="s">
+        <v>258</v>
+      </c>
+      <c r="C86" t="s">
+        <v>259</v>
+      </c>
+      <c r="D86">
+        <v>11</v>
+      </c>
+      <c r="E86">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5">
+      <c r="A87">
+        <v>86</v>
+      </c>
+      <c r="B87" t="s">
+        <v>260</v>
+      </c>
+      <c r="C87" t="s">
+        <v>261</v>
+      </c>
+      <c r="D87">
+        <v>11</v>
+      </c>
+      <c r="E87">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5">
+      <c r="A88">
+        <v>87</v>
+      </c>
+      <c r="B88" t="s">
+        <v>262</v>
+      </c>
+      <c r="C88" t="s">
+        <v>263</v>
+      </c>
+      <c r="D88">
+        <v>11</v>
+      </c>
+      <c r="E88">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5">
+      <c r="A89">
+        <v>88</v>
+      </c>
+      <c r="B89" t="s">
+        <v>264</v>
+      </c>
+      <c r="C89" t="s">
+        <v>265</v>
+      </c>
+      <c r="D89">
+        <v>12</v>
+      </c>
+      <c r="E89">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5">
+      <c r="A90">
+        <v>89</v>
+      </c>
+      <c r="B90" t="s">
+        <v>266</v>
+      </c>
+      <c r="C90" t="s">
+        <v>267</v>
+      </c>
+      <c r="D90">
+        <v>12</v>
+      </c>
+      <c r="E90">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5">
+      <c r="A91">
+        <v>90</v>
+      </c>
+      <c r="B91" t="s">
+        <v>268</v>
+      </c>
+      <c r="C91" t="s">
+        <v>269</v>
+      </c>
+      <c r="D91">
+        <v>12</v>
+      </c>
+      <c r="E91">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5">
+      <c r="A92">
+        <v>91</v>
+      </c>
+      <c r="B92" t="s">
+        <v>270</v>
+      </c>
+      <c r="C92" t="s">
+        <v>271</v>
+      </c>
+      <c r="D92">
+        <v>14</v>
+      </c>
+      <c r="E92">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5">
+      <c r="A93">
+        <v>92</v>
+      </c>
+      <c r="B93" t="s">
+        <v>272</v>
+      </c>
+      <c r="C93" t="s">
+        <v>273</v>
+      </c>
+      <c r="D93">
+        <v>14</v>
+      </c>
+      <c r="E93">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5">
+      <c r="A94">
+        <v>93</v>
+      </c>
+      <c r="B94" t="s">
+        <v>274</v>
+      </c>
+      <c r="C94" t="s">
+        <v>275</v>
+      </c>
+      <c r="D94">
+        <v>13</v>
+      </c>
+      <c r="E94">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5">
+      <c r="A95">
+        <v>94</v>
+      </c>
+      <c r="B95" t="s">
+        <v>276</v>
+      </c>
+      <c r="C95" t="s">
+        <v>277</v>
+      </c>
+      <c r="D95">
+        <v>13</v>
+      </c>
+      <c r="E95">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5">
+      <c r="A96">
+        <v>95</v>
+      </c>
+      <c r="B96" t="s">
+        <v>278</v>
+      </c>
+      <c r="C96" t="s">
+        <v>279</v>
+      </c>
+      <c r="D96">
+        <v>15</v>
+      </c>
+      <c r="E96">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5">
+      <c r="A97">
+        <v>96</v>
+      </c>
+      <c r="B97" t="s">
+        <v>280</v>
+      </c>
+      <c r="C97" t="s">
+        <v>279</v>
+      </c>
+      <c r="D97">
+        <v>15</v>
+      </c>
+      <c r="E97">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5">
+      <c r="A98">
+        <v>97</v>
+      </c>
+      <c r="B98" t="s">
+        <v>281</v>
+      </c>
+      <c r="C98" t="s">
+        <v>282</v>
+      </c>
+      <c r="D98">
+        <v>16</v>
+      </c>
+      <c r="E98">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5">
+      <c r="A99">
+        <v>98</v>
+      </c>
+      <c r="B99" t="s">
+        <v>283</v>
+      </c>
+      <c r="C99" t="s">
+        <v>284</v>
+      </c>
+      <c r="D99">
+        <v>16</v>
+      </c>
+      <c r="E99">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5">
+      <c r="A100">
+        <v>99</v>
+      </c>
+      <c r="B100" t="s">
+        <v>285</v>
+      </c>
+      <c r="C100" t="s">
+        <v>286</v>
+      </c>
+      <c r="D100">
+        <v>20</v>
+      </c>
+      <c r="E100">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5">
+      <c r="A101">
+        <v>100</v>
+      </c>
+      <c r="B101" t="s">
+        <v>287</v>
+      </c>
+      <c r="C101" t="s">
+        <v>288</v>
+      </c>
+      <c r="D101">
+        <v>20</v>
+      </c>
+      <c r="E101">
+        <v>11</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B485A97C-E092-4E06-B68C-90ECE5645DB1}">
+  <dimension ref="A1:E101"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="4" max="4" width="16" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>289</v>
+      </c>
+      <c r="C1" t="s">
+        <v>290</v>
+      </c>
+      <c r="D1" t="s">
+        <v>291</v>
+      </c>
+      <c r="E1" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>12000</v>
+      </c>
+      <c r="C2" t="s">
+        <v>293</v>
+      </c>
+      <c r="D2">
+        <v>150</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>13000</v>
+      </c>
+      <c r="C3" t="s">
+        <v>293</v>
+      </c>
+      <c r="D3">
+        <v>140</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>14000</v>
+      </c>
+      <c r="C4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D4">
+        <v>120</v>
+      </c>
+      <c r="E4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>10000</v>
+      </c>
+      <c r="C5" t="s">
+        <v>295</v>
+      </c>
+      <c r="D5">
+        <v>300</v>
+      </c>
+      <c r="E5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>10000</v>
+      </c>
+      <c r="C6" t="s">
+        <v>295</v>
+      </c>
+      <c r="D6">
+        <v>250</v>
+      </c>
+      <c r="E6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>10000</v>
+      </c>
+      <c r="C7" t="s">
+        <v>295</v>
+      </c>
+      <c r="D7">
+        <v>280</v>
+      </c>
+      <c r="E7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>12000</v>
+      </c>
+      <c r="C8" t="s">
+        <v>295</v>
+      </c>
+      <c r="D8">
+        <v>180</v>
+      </c>
+      <c r="E8">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>15000</v>
+      </c>
+      <c r="C9" t="s">
+        <v>295</v>
+      </c>
+      <c r="D9">
+        <v>160</v>
+      </c>
+      <c r="E9">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>18000</v>
+      </c>
+      <c r="C10" t="s">
+        <v>296</v>
+      </c>
+      <c r="D10">
+        <v>100</v>
+      </c>
+      <c r="E10">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>18000</v>
+      </c>
+      <c r="C11" t="s">
+        <v>296</v>
+      </c>
+      <c r="D11">
+        <v>100</v>
+      </c>
+      <c r="E11">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12">
+        <v>35000</v>
+      </c>
+      <c r="C12" t="s">
+        <v>294</v>
+      </c>
+      <c r="D12">
+        <v>80</v>
+      </c>
+      <c r="E12">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13">
+        <v>28000</v>
+      </c>
+      <c r="C13" t="s">
+        <v>294</v>
+      </c>
+      <c r="D13">
+        <v>90</v>
+      </c>
+      <c r="E13">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14">
+        <v>45000</v>
+      </c>
+      <c r="C14" t="s">
+        <v>294</v>
+      </c>
+      <c r="D14">
+        <v>60</v>
+      </c>
+      <c r="E14">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15">
+        <v>5000</v>
+      </c>
+      <c r="C15" t="s">
+        <v>297</v>
+      </c>
+      <c r="D15">
+        <v>400</v>
+      </c>
+      <c r="E15">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16">
+        <v>8000</v>
+      </c>
+      <c r="C16" t="s">
+        <v>297</v>
+      </c>
+      <c r="D16">
+        <v>300</v>
+      </c>
+      <c r="E16">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17">
+        <v>4500</v>
+      </c>
+      <c r="C17" t="s">
+        <v>297</v>
+      </c>
+      <c r="D17">
+        <v>350</v>
+      </c>
+      <c r="E17">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18">
+        <v>9000</v>
+      </c>
+      <c r="C18" t="s">
+        <v>297</v>
+      </c>
+      <c r="D18">
+        <v>250</v>
+      </c>
+      <c r="E18">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19">
+        <v>22000</v>
+      </c>
+      <c r="C19" t="s">
+        <v>296</v>
+      </c>
+      <c r="D19">
+        <v>120</v>
+      </c>
+      <c r="E19">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20">
+        <v>22000</v>
+      </c>
+      <c r="C20" t="s">
+        <v>296</v>
+      </c>
+      <c r="D20">
+        <v>120</v>
+      </c>
+      <c r="E20">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21">
+        <v>55000</v>
+      </c>
+      <c r="C21" t="s">
+        <v>295</v>
+      </c>
+      <c r="D21">
+        <v>70</v>
+      </c>
+      <c r="E21">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22">
+        <v>20000</v>
+      </c>
+      <c r="C22" t="s">
+        <v>296</v>
+      </c>
+      <c r="D22">
+        <v>90</v>
+      </c>
+      <c r="E22">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23">
+        <v>45000</v>
+      </c>
+      <c r="C23" t="s">
+        <v>294</v>
+      </c>
+      <c r="D23">
+        <v>150</v>
+      </c>
+      <c r="E23">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24">
+        <v>22000</v>
+      </c>
+      <c r="C24" t="s">
+        <v>295</v>
+      </c>
+      <c r="D24">
+        <v>120</v>
+      </c>
+      <c r="E24">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25">
+        <v>10000</v>
+      </c>
+      <c r="C25" t="s">
+        <v>293</v>
+      </c>
+      <c r="D25">
+        <v>220</v>
+      </c>
+      <c r="E25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26">
+        <v>12000</v>
+      </c>
+      <c r="C26" t="s">
+        <v>295</v>
+      </c>
+      <c r="D26">
+        <v>150</v>
+      </c>
+      <c r="E26">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27">
+        <v>12000</v>
+      </c>
+      <c r="C27" t="s">
+        <v>295</v>
+      </c>
+      <c r="D27">
+        <v>180</v>
+      </c>
+      <c r="E27">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28">
+        <v>7000</v>
+      </c>
+      <c r="C28" t="s">
+        <v>293</v>
+      </c>
+      <c r="D28">
+        <v>500</v>
+      </c>
+      <c r="E28">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29">
+        <v>7000</v>
+      </c>
+      <c r="C29" t="s">
+        <v>293</v>
+      </c>
+      <c r="D29">
+        <v>500</v>
+      </c>
+      <c r="E29">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30">
+        <v>5000</v>
+      </c>
+      <c r="C30" t="s">
+        <v>297</v>
+      </c>
+      <c r="D30">
+        <v>300</v>
+      </c>
+      <c r="E30">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31">
+        <v>36000</v>
+      </c>
+      <c r="C31" t="s">
+        <v>294</v>
+      </c>
+      <c r="D31">
+        <v>80</v>
+      </c>
+      <c r="E31">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32">
+        <v>18000</v>
+      </c>
+      <c r="C32" t="s">
+        <v>297</v>
+      </c>
+      <c r="D32">
+        <v>140</v>
+      </c>
+      <c r="E32">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33">
+        <v>12000</v>
+      </c>
+      <c r="C33" t="s">
+        <v>297</v>
+      </c>
+      <c r="D33">
+        <v>160</v>
+      </c>
+      <c r="E33">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34">
+        <v>15000</v>
+      </c>
+      <c r="C34" t="s">
+        <v>297</v>
+      </c>
+      <c r="D34">
+        <v>170</v>
+      </c>
+      <c r="E34">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35">
+        <v>13000</v>
+      </c>
+      <c r="C35" t="s">
+        <v>293</v>
+      </c>
+      <c r="D35">
+        <v>120</v>
+      </c>
+      <c r="E35">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36">
+        <v>15000</v>
+      </c>
+      <c r="C36" t="s">
+        <v>294</v>
+      </c>
+      <c r="D36">
+        <v>110</v>
+      </c>
+      <c r="E36">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37">
+        <v>12000</v>
+      </c>
+      <c r="C37" t="s">
+        <v>295</v>
+      </c>
+      <c r="D37">
+        <v>200</v>
+      </c>
+      <c r="E37">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38">
+        <v>12000</v>
+      </c>
+      <c r="C38" t="s">
+        <v>295</v>
+      </c>
+      <c r="D38">
+        <v>180</v>
+      </c>
+      <c r="E38">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5">
+      <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39">
+        <v>16000</v>
+      </c>
+      <c r="C39" t="s">
+        <v>295</v>
+      </c>
+      <c r="D39">
+        <v>120</v>
+      </c>
+      <c r="E39">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40">
+        <v>18000</v>
+      </c>
+      <c r="C40" t="s">
+        <v>296</v>
+      </c>
+      <c r="D40">
+        <v>100</v>
+      </c>
+      <c r="E40">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41">
+        <v>35000</v>
+      </c>
+      <c r="C41" t="s">
+        <v>294</v>
+      </c>
+      <c r="D41">
+        <v>80</v>
+      </c>
+      <c r="E41">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5">
+      <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42">
+        <v>6000</v>
+      </c>
+      <c r="C42" t="s">
+        <v>297</v>
+      </c>
+      <c r="D42">
+        <v>250</v>
+      </c>
+      <c r="E42">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43">
+        <v>9000</v>
+      </c>
+      <c r="C43" t="s">
+        <v>297</v>
+      </c>
+      <c r="D43">
+        <v>240</v>
+      </c>
+      <c r="E43">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5">
+      <c r="A44">
+        <v>43</v>
+      </c>
+      <c r="B44">
+        <v>5000</v>
+      </c>
+      <c r="C44" t="s">
+        <v>297</v>
+      </c>
+      <c r="D44">
+        <v>260</v>
+      </c>
+      <c r="E44">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5">
+      <c r="A45">
+        <v>44</v>
+      </c>
+      <c r="B45">
+        <v>10000</v>
+      </c>
+      <c r="C45" t="s">
+        <v>297</v>
+      </c>
+      <c r="D45">
+        <v>180</v>
+      </c>
+      <c r="E45">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5">
+      <c r="A46">
+        <v>45</v>
+      </c>
+      <c r="B46">
+        <v>22000</v>
+      </c>
+      <c r="C46" t="s">
+        <v>296</v>
+      </c>
+      <c r="D46">
+        <v>120</v>
+      </c>
+      <c r="E46">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5">
+      <c r="A47">
+        <v>46</v>
+      </c>
+      <c r="B47">
+        <v>55000</v>
+      </c>
+      <c r="C47" t="s">
+        <v>295</v>
+      </c>
+      <c r="D47">
+        <v>70</v>
+      </c>
+      <c r="E47">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5">
+      <c r="A48">
+        <v>47</v>
+      </c>
+      <c r="B48">
+        <v>18000</v>
+      </c>
+      <c r="C48" t="s">
+        <v>296</v>
+      </c>
+      <c r="D48">
+        <v>90</v>
+      </c>
+      <c r="E48">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5">
+      <c r="A49">
+        <v>48</v>
+      </c>
+      <c r="B49">
+        <v>50000</v>
+      </c>
+      <c r="C49" t="s">
+        <v>294</v>
+      </c>
+      <c r="D49">
+        <v>100</v>
+      </c>
+      <c r="E49">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5">
+      <c r="A50">
+        <v>49</v>
+      </c>
+      <c r="B50">
+        <v>24000</v>
+      </c>
+      <c r="C50" t="s">
+        <v>295</v>
+      </c>
+      <c r="D50">
+        <v>110</v>
+      </c>
+      <c r="E50">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5">
+      <c r="A51">
+        <v>50</v>
+      </c>
+      <c r="B51">
+        <v>10000</v>
+      </c>
+      <c r="C51" t="s">
+        <v>293</v>
+      </c>
+      <c r="D51">
+        <v>210</v>
+      </c>
+      <c r="E51">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5">
+      <c r="A52">
+        <v>51</v>
+      </c>
+      <c r="B52">
+        <v>12000</v>
+      </c>
+      <c r="C52" t="s">
+        <v>295</v>
+      </c>
+      <c r="D52">
+        <v>150</v>
+      </c>
+      <c r="E52">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5">
+      <c r="A53">
+        <v>52</v>
+      </c>
+      <c r="B53">
+        <v>14000</v>
+      </c>
+      <c r="C53" t="s">
+        <v>295</v>
+      </c>
+      <c r="D53">
+        <v>130</v>
+      </c>
+      <c r="E53">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5">
+      <c r="A54">
+        <v>53</v>
+      </c>
+      <c r="B54">
+        <v>9000</v>
+      </c>
+      <c r="C54" t="s">
+        <v>293</v>
+      </c>
+      <c r="D54">
+        <v>200</v>
+      </c>
+      <c r="E54">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5">
+      <c r="A55">
+        <v>54</v>
+      </c>
+      <c r="B55">
+        <v>9000</v>
+      </c>
+      <c r="C55" t="s">
+        <v>293</v>
+      </c>
+      <c r="D55">
+        <v>180</v>
+      </c>
+      <c r="E55">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5">
+      <c r="A56">
+        <v>55</v>
+      </c>
+      <c r="B56">
+        <v>20000</v>
+      </c>
+      <c r="C56" t="s">
+        <v>297</v>
+      </c>
+      <c r="D56">
+        <v>100</v>
+      </c>
+      <c r="E56">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5">
+      <c r="A57">
+        <v>56</v>
+      </c>
+      <c r="B57">
+        <v>12000</v>
+      </c>
+      <c r="C57" t="s">
+        <v>297</v>
+      </c>
+      <c r="D57">
+        <v>120</v>
+      </c>
+      <c r="E57">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5">
+      <c r="A58">
+        <v>57</v>
+      </c>
+      <c r="B58">
+        <v>15000</v>
+      </c>
+      <c r="C58" t="s">
+        <v>297</v>
+      </c>
+      <c r="D58">
+        <v>110</v>
+      </c>
+      <c r="E58">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5">
+      <c r="A59">
+        <v>58</v>
+      </c>
+      <c r="B59">
+        <v>18000</v>
+      </c>
+      <c r="C59" t="s">
+        <v>298</v>
+      </c>
+      <c r="D59">
+        <v>50</v>
+      </c>
+      <c r="E59">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5">
+      <c r="A60">
+        <v>59</v>
+      </c>
+      <c r="B60">
+        <v>22000</v>
+      </c>
+      <c r="C60" t="s">
+        <v>298</v>
+      </c>
+      <c r="D60">
+        <v>40</v>
+      </c>
+      <c r="E60">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5">
+      <c r="A61">
+        <v>60</v>
+      </c>
+      <c r="B61">
+        <v>35000</v>
+      </c>
+      <c r="C61" t="s">
+        <v>298</v>
+      </c>
+      <c r="D61">
+        <v>35</v>
+      </c>
+      <c r="E61">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5">
+      <c r="A62">
+        <v>61</v>
+      </c>
+      <c r="B62">
+        <v>42000</v>
+      </c>
+      <c r="C62" t="s">
+        <v>294</v>
+      </c>
+      <c r="D62">
+        <v>30</v>
+      </c>
+      <c r="E62">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5">
+      <c r="A63">
+        <v>62</v>
+      </c>
+      <c r="B63">
+        <v>42000</v>
+      </c>
+      <c r="C63" t="s">
+        <v>294</v>
+      </c>
+      <c r="D63">
+        <v>25</v>
+      </c>
+      <c r="E63">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5">
+      <c r="A64">
+        <v>63</v>
+      </c>
+      <c r="B64">
+        <v>28000</v>
+      </c>
+      <c r="C64" t="s">
+        <v>297</v>
+      </c>
+      <c r="D64">
+        <v>60</v>
+      </c>
+      <c r="E64">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5">
+      <c r="A65">
+        <v>64</v>
+      </c>
+      <c r="B65">
+        <v>85000</v>
+      </c>
+      <c r="C65" t="s">
+        <v>296</v>
+      </c>
+      <c r="D65">
+        <v>20</v>
+      </c>
+      <c r="E65">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5">
+      <c r="A66">
+        <v>65</v>
+      </c>
+      <c r="B66">
+        <v>45000</v>
+      </c>
+      <c r="C66" t="s">
+        <v>299</v>
+      </c>
+      <c r="D66">
+        <v>40</v>
+      </c>
+      <c r="E66">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5">
+      <c r="A67">
+        <v>66</v>
+      </c>
+      <c r="B67">
+        <v>45000</v>
+      </c>
+      <c r="C67" t="s">
+        <v>299</v>
+      </c>
+      <c r="D67">
+        <v>40</v>
+      </c>
+      <c r="E67">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5">
+      <c r="A68">
+        <v>67</v>
+      </c>
+      <c r="B68">
+        <v>25000</v>
+      </c>
+      <c r="C68" t="s">
+        <v>300</v>
+      </c>
+      <c r="D68">
+        <v>50</v>
+      </c>
+      <c r="E68">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5">
+      <c r="A69">
+        <v>68</v>
+      </c>
+      <c r="B69">
+        <v>30000</v>
+      </c>
+      <c r="C69" t="s">
+        <v>300</v>
+      </c>
+      <c r="D69">
+        <v>60</v>
+      </c>
+      <c r="E69">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5">
+      <c r="A70">
+        <v>69</v>
+      </c>
+      <c r="B70">
+        <v>45000</v>
+      </c>
+      <c r="C70" t="s">
+        <v>300</v>
+      </c>
+      <c r="D70">
+        <v>40</v>
+      </c>
+      <c r="E70">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5">
+      <c r="A71">
+        <v>70</v>
+      </c>
+      <c r="B71">
+        <v>18000</v>
+      </c>
+      <c r="C71" t="s">
+        <v>298</v>
+      </c>
+      <c r="D71">
+        <v>45</v>
+      </c>
+      <c r="E71">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5">
+      <c r="A72">
+        <v>71</v>
+      </c>
+      <c r="B72">
+        <v>95000</v>
+      </c>
+      <c r="C72" t="s">
+        <v>300</v>
+      </c>
+      <c r="D72">
+        <v>35</v>
+      </c>
+      <c r="E72">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5">
+      <c r="A73">
+        <v>72</v>
+      </c>
+      <c r="B73">
+        <v>140000</v>
+      </c>
+      <c r="C73" t="s">
+        <v>300</v>
+      </c>
+      <c r="D73">
+        <v>25</v>
+      </c>
+      <c r="E73">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5">
+      <c r="A74">
+        <v>73</v>
+      </c>
+      <c r="B74">
+        <v>38000</v>
+      </c>
+      <c r="C74" t="s">
+        <v>297</v>
+      </c>
+      <c r="D74">
+        <v>80</v>
+      </c>
+      <c r="E74">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5">
+      <c r="A75">
+        <v>74</v>
+      </c>
+      <c r="B75">
+        <v>25000</v>
+      </c>
+      <c r="C75" t="s">
+        <v>298</v>
+      </c>
+      <c r="D75">
+        <v>60</v>
+      </c>
+      <c r="E75">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5">
+      <c r="A76">
+        <v>75</v>
+      </c>
+      <c r="B76">
+        <v>18000</v>
+      </c>
+      <c r="C76" t="s">
+        <v>298</v>
+      </c>
+      <c r="D76">
+        <v>50</v>
+      </c>
+      <c r="E76">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5">
+      <c r="A77">
+        <v>76</v>
+      </c>
+      <c r="B77">
+        <v>30000</v>
+      </c>
+      <c r="C77" t="s">
+        <v>298</v>
+      </c>
+      <c r="D77">
+        <v>35</v>
+      </c>
+      <c r="E77">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5">
+      <c r="A78">
+        <v>77</v>
+      </c>
+      <c r="B78">
+        <v>22000</v>
+      </c>
+      <c r="C78" t="s">
+        <v>294</v>
+      </c>
+      <c r="D78">
+        <v>90</v>
+      </c>
+      <c r="E78">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5">
+      <c r="A79">
+        <v>78</v>
+      </c>
+      <c r="B79">
+        <v>18000</v>
+      </c>
+      <c r="C79" t="s">
+        <v>301</v>
+      </c>
+      <c r="D79">
+        <v>120</v>
+      </c>
+      <c r="E79">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5">
+      <c r="A80">
+        <v>79</v>
+      </c>
+      <c r="B80">
+        <v>20000</v>
+      </c>
+      <c r="C80" t="s">
+        <v>301</v>
+      </c>
+      <c r="D80">
+        <v>100</v>
+      </c>
+      <c r="E80">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5">
+      <c r="A81">
+        <v>80</v>
+      </c>
+      <c r="B81">
+        <v>42000</v>
+      </c>
+      <c r="C81" t="s">
+        <v>295</v>
+      </c>
+      <c r="D81">
+        <v>80</v>
+      </c>
+      <c r="E81">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5">
+      <c r="A82">
+        <v>81</v>
+      </c>
+      <c r="B82">
+        <v>38000</v>
+      </c>
+      <c r="C82" t="s">
+        <v>295</v>
+      </c>
+      <c r="D82">
+        <v>80</v>
+      </c>
+      <c r="E82">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5">
+      <c r="A83">
+        <v>82</v>
+      </c>
+      <c r="B83">
+        <v>35000</v>
+      </c>
+      <c r="C83" t="s">
+        <v>295</v>
+      </c>
+      <c r="D83">
+        <v>60</v>
+      </c>
+      <c r="E83">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5">
+      <c r="A84">
+        <v>83</v>
+      </c>
+      <c r="B84">
+        <v>28000</v>
+      </c>
+      <c r="C84" t="s">
+        <v>293</v>
+      </c>
+      <c r="D84">
+        <v>70</v>
+      </c>
+      <c r="E84">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5">
+      <c r="A85">
+        <v>84</v>
+      </c>
+      <c r="B85">
+        <v>32000</v>
+      </c>
+      <c r="C85" t="s">
+        <v>293</v>
+      </c>
+      <c r="D85">
+        <v>60</v>
+      </c>
+      <c r="E85">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5">
+      <c r="A86">
+        <v>85</v>
+      </c>
+      <c r="B86">
+        <v>75000</v>
+      </c>
+      <c r="C86" t="s">
+        <v>293</v>
+      </c>
+      <c r="D86">
+        <v>40</v>
+      </c>
+      <c r="E86">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5">
+      <c r="A87">
+        <v>86</v>
+      </c>
+      <c r="B87">
+        <v>85000</v>
+      </c>
+      <c r="C87" t="s">
+        <v>293</v>
+      </c>
+      <c r="D87">
+        <v>35</v>
+      </c>
+      <c r="E87">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5">
+      <c r="A88">
+        <v>87</v>
+      </c>
+      <c r="B88">
+        <v>42000</v>
+      </c>
+      <c r="C88" t="s">
+        <v>294</v>
+      </c>
+      <c r="D88">
+        <v>70</v>
+      </c>
+      <c r="E88">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5">
+      <c r="A89">
+        <v>88</v>
+      </c>
+      <c r="B89">
+        <v>120000</v>
+      </c>
+      <c r="C89" t="s">
+        <v>293</v>
+      </c>
+      <c r="D89">
+        <v>30</v>
+      </c>
+      <c r="E89">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5">
+      <c r="A90">
+        <v>89</v>
+      </c>
+      <c r="B90">
+        <v>38000</v>
+      </c>
+      <c r="C90" t="s">
+        <v>293</v>
+      </c>
+      <c r="D90">
+        <v>50</v>
+      </c>
+      <c r="E90">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5">
+      <c r="A91">
+        <v>90</v>
+      </c>
+      <c r="B91">
+        <v>28000</v>
+      </c>
+      <c r="C91" t="s">
+        <v>294</v>
+      </c>
+      <c r="D91">
+        <v>100</v>
+      </c>
+      <c r="E91">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5">
+      <c r="A92">
+        <v>91</v>
+      </c>
+      <c r="B92">
+        <v>90000</v>
+      </c>
+      <c r="C92" t="s">
+        <v>296</v>
+      </c>
+      <c r="D92">
+        <v>20</v>
+      </c>
+      <c r="E92">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5">
+      <c r="A93">
+        <v>92</v>
+      </c>
+      <c r="B93">
+        <v>150000</v>
+      </c>
+      <c r="C93" t="s">
+        <v>296</v>
+      </c>
+      <c r="D93">
+        <v>15</v>
+      </c>
+      <c r="E93">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5">
+      <c r="A94">
+        <v>93</v>
+      </c>
+      <c r="B94">
+        <v>320000</v>
+      </c>
+      <c r="C94" t="s">
+        <v>297</v>
+      </c>
+      <c r="D94">
+        <v>20</v>
+      </c>
+      <c r="E94">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5">
+      <c r="A95">
+        <v>94</v>
+      </c>
+      <c r="B95">
+        <v>45000</v>
+      </c>
+      <c r="C95" t="s">
+        <v>297</v>
+      </c>
+      <c r="D95">
+        <v>50</v>
+      </c>
+      <c r="E95">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5">
+      <c r="A96">
+        <v>95</v>
+      </c>
+      <c r="B96">
+        <v>35000</v>
+      </c>
+      <c r="C96" t="s">
+        <v>297</v>
+      </c>
+      <c r="D96">
+        <v>100</v>
+      </c>
+      <c r="E96">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5">
+      <c r="A97">
+        <v>96</v>
+      </c>
+      <c r="B97">
+        <v>38000</v>
+      </c>
+      <c r="C97" t="s">
+        <v>297</v>
+      </c>
+      <c r="D97">
+        <v>90</v>
+      </c>
+      <c r="E97">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5">
+      <c r="A98">
+        <v>97</v>
+      </c>
+      <c r="B98">
+        <v>22000</v>
+      </c>
+      <c r="C98" t="s">
+        <v>295</v>
+      </c>
+      <c r="D98">
+        <v>150</v>
+      </c>
+      <c r="E98">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5">
+      <c r="A99">
+        <v>98</v>
+      </c>
+      <c r="B99">
+        <v>28000</v>
+      </c>
+      <c r="C99" t="s">
+        <v>293</v>
+      </c>
+      <c r="D99">
+        <v>120</v>
+      </c>
+      <c r="E99">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5">
+      <c r="A100">
+        <v>99</v>
+      </c>
+      <c r="B100">
+        <v>85000</v>
+      </c>
+      <c r="C100" t="s">
+        <v>294</v>
+      </c>
+      <c r="D100">
+        <v>30</v>
+      </c>
+      <c r="E100">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5">
+      <c r="A101">
+        <v>100</v>
+      </c>
+      <c r="B101">
+        <v>150000</v>
+      </c>
+      <c r="C101" t="s">
+        <v>294</v>
+      </c>
+      <c r="D101">
+        <v>20</v>
+      </c>
+      <c r="E101">
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Refactor brands, add image entities, update seeder
- Refactored BrandsController for attribute-based binding and simplified action results
- Updated CreateBrandCommandHandler and BrandRepository constructors
- Removed case-insensitive comparison in FindNameAsync methods
- Split Entity class; moved AuditableEntity and SoftDeletableEntity to separate files
- Added Image and ProductImage domain entities with configurations
- Switched to UseIdentityByDefaultColumn for PostgreSQL compatibility
- Enhanced database seeder to sync Postgres sequences after seeding
- Updated ConvenienceStoreData.xlsx data file
</commit_message>
<xml_diff>
--- a/src/External/ConvenienceStore.Persistence/Data/ConvenienceStoreData.xlsx
+++ b/src/External/ConvenienceStore.Persistence/Data/ConvenienceStoreData.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30318"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30317"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="50" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0002D883-D255-43C5-BD49-3325098AB764}"/>
+  <xr:revisionPtr revIDLastSave="55" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{36C8C329-DFE6-4DAB-B9AC-212ABB5056D7}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Categories" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="302">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="418" uniqueCount="304">
   <si>
     <t>Id</t>
   </si>
@@ -372,6 +372,12 @@
   </si>
   <si>
     <t>Thương hiệu kẹo sữa và caramel được ưa chuộng tại Việt Nam.</t>
+  </si>
+  <si>
+    <t>Otoki</t>
+  </si>
+  <si>
+    <t>Otoki Việt Nam mang chất lượng chuẩn Hàn Quốc từ thương hiệu uy tín ra đời năm 1969.</t>
   </si>
   <si>
     <t>CategoryId</t>
@@ -1572,7 +1578,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{748F4E0F-BC34-4228-867E-9D0F821705DC}">
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1914,6 +1920,17 @@
       </c>
       <c r="C31" t="s">
         <v>102</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="s">
+        <v>103</v>
+      </c>
+      <c r="C32" t="s">
+        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -1926,6 +1943,7 @@
   <dimension ref="A1:E101"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
+    <col min="2" max="2" width="28" customWidth="1"/>
     <col min="3" max="3" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.5703125" bestFit="1" customWidth="1"/>
   </cols>
@@ -1941,10 +1959,10 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E1" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -1952,10 +1970,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C2" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -1969,10 +1987,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C3" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D3">
         <v>1</v>
@@ -1986,10 +2004,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C4" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -2003,10 +2021,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -2020,10 +2038,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -2037,10 +2055,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C7" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -2054,10 +2072,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C8" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D8">
         <v>1</v>
@@ -2071,10 +2089,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C9" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -2088,10 +2106,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C10" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D10">
         <v>2</v>
@@ -2105,10 +2123,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C11" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D11">
         <v>2</v>
@@ -2122,10 +2140,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C12" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D12">
         <v>10</v>
@@ -2139,10 +2157,10 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C13" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="D13">
         <v>5</v>
@@ -2156,10 +2174,10 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C14" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D14">
         <v>10</v>
@@ -2173,10 +2191,10 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C15" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D15">
         <v>3</v>
@@ -2190,10 +2208,10 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C16" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D16">
         <v>3</v>
@@ -2207,10 +2225,10 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C17" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D17">
         <v>3</v>
@@ -2224,10 +2242,10 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C18" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D18">
         <v>3</v>
@@ -2241,10 +2259,10 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C19" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D19">
         <v>2</v>
@@ -2258,10 +2276,10 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C20" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D20">
         <v>2</v>
@@ -2275,10 +2293,10 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C21" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D21">
         <v>2</v>
@@ -2292,10 +2310,10 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C22" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D22">
         <v>2</v>
@@ -2309,10 +2327,10 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C23" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D23">
         <v>1</v>
@@ -2326,10 +2344,10 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C24" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D24">
         <v>1</v>
@@ -2343,10 +2361,10 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C25" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D25">
         <v>1</v>
@@ -2360,10 +2378,10 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C26" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D26">
         <v>1</v>
@@ -2377,10 +2395,10 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C27" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D27">
         <v>1</v>
@@ -2394,10 +2412,10 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C28" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D28">
         <v>1</v>
@@ -2411,10 +2429,10 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C29" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D29">
         <v>1</v>
@@ -2428,10 +2446,10 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C30" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D30">
         <v>3</v>
@@ -2445,10 +2463,10 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C31" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="D31">
         <v>10</v>
@@ -2462,10 +2480,10 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C32" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="D32">
         <v>10</v>
@@ -2479,10 +2497,10 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C33" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D33">
         <v>10</v>
@@ -2496,10 +2514,10 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="C34" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D34">
         <v>10</v>
@@ -2513,10 +2531,10 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C35" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D35">
         <v>1</v>
@@ -2530,10 +2548,10 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C36" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D36">
         <v>1</v>
@@ -2547,10 +2565,10 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C37" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="D37">
         <v>1</v>
@@ -2564,10 +2582,10 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C38" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D38">
         <v>1</v>
@@ -2581,10 +2599,10 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C39" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D39">
         <v>1</v>
@@ -2598,10 +2616,10 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="C40" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="D40">
         <v>2</v>
@@ -2615,10 +2633,10 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="C41" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="D41">
         <v>10</v>
@@ -2632,10 +2650,10 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C42" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D42">
         <v>3</v>
@@ -2649,16 +2667,16 @@
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C43" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="D43">
         <v>3</v>
       </c>
       <c r="E43">
-        <v>13</v>
+        <v>31</v>
       </c>
     </row>
     <row r="44" spans="1:5">
@@ -2666,10 +2684,10 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C44" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D44">
         <v>3</v>
@@ -2683,10 +2701,10 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="C45" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="D45">
         <v>3</v>
@@ -2700,10 +2718,10 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C46" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D46">
         <v>2</v>
@@ -2717,10 +2735,10 @@
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C47" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D47">
         <v>2</v>
@@ -2734,10 +2752,10 @@
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="C48" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="D48">
         <v>2</v>
@@ -2751,10 +2769,10 @@
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C49" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="D49">
         <v>1</v>
@@ -2768,10 +2786,10 @@
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="C50" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="D50">
         <v>1</v>
@@ -2785,10 +2803,10 @@
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C51" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D51">
         <v>1</v>
@@ -2802,10 +2820,10 @@
         <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C52" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="D52">
         <v>1</v>
@@ -2819,10 +2837,10 @@
         <v>52</v>
       </c>
       <c r="B53" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C53" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D53">
         <v>1</v>
@@ -2836,10 +2854,10 @@
         <v>53</v>
       </c>
       <c r="B54" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C54" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D54">
         <v>1</v>
@@ -2853,10 +2871,10 @@
         <v>54</v>
       </c>
       <c r="B55" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C55" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D55">
         <v>1</v>
@@ -2870,10 +2888,10 @@
         <v>55</v>
       </c>
       <c r="B56" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C56" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="D56">
         <v>10</v>
@@ -2887,10 +2905,10 @@
         <v>56</v>
       </c>
       <c r="B57" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C57" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="D57">
         <v>10</v>
@@ -2904,10 +2922,10 @@
         <v>57</v>
       </c>
       <c r="B58" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="C58" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="D58">
         <v>10</v>
@@ -2921,10 +2939,10 @@
         <v>58</v>
       </c>
       <c r="B59" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="C59" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="D59">
         <v>5</v>
@@ -2938,10 +2956,10 @@
         <v>59</v>
       </c>
       <c r="B60" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="C60" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="D60">
         <v>5</v>
@@ -2955,10 +2973,10 @@
         <v>60</v>
       </c>
       <c r="B61" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="C61" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D61">
         <v>17</v>
@@ -2972,10 +2990,10 @@
         <v>61</v>
       </c>
       <c r="B62" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C62" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D62">
         <v>17</v>
@@ -2989,10 +3007,10 @@
         <v>62</v>
       </c>
       <c r="B63" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C63" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D63">
         <v>17</v>
@@ -3006,10 +3024,10 @@
         <v>63</v>
       </c>
       <c r="B64" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="C64" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D64">
         <v>8</v>
@@ -3023,10 +3041,10 @@
         <v>64</v>
       </c>
       <c r="B65" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="C65" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="D65">
         <v>6</v>
@@ -3040,10 +3058,10 @@
         <v>65</v>
       </c>
       <c r="B66" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="C66" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D66">
         <v>19</v>
@@ -3057,10 +3075,10 @@
         <v>66</v>
       </c>
       <c r="B67" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="C67" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="D67">
         <v>19</v>
@@ -3074,10 +3092,10 @@
         <v>67</v>
       </c>
       <c r="B68" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C68" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="D68">
         <v>7</v>
@@ -3091,10 +3109,10 @@
         <v>68</v>
       </c>
       <c r="B69" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="C69" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="D69">
         <v>7</v>
@@ -3108,10 +3126,10 @@
         <v>69</v>
       </c>
       <c r="B70" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="C70" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="D70">
         <v>7</v>
@@ -3125,10 +3143,10 @@
         <v>70</v>
       </c>
       <c r="B71" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="C71" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="D71">
         <v>7</v>
@@ -3142,10 +3160,10 @@
         <v>71</v>
       </c>
       <c r="B72" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="C72" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D72">
         <v>8</v>
@@ -3159,10 +3177,10 @@
         <v>72</v>
       </c>
       <c r="B73" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C73" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="D73">
         <v>8</v>
@@ -3176,10 +3194,10 @@
         <v>73</v>
       </c>
       <c r="B74" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="C74" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="D74">
         <v>4</v>
@@ -3193,10 +3211,10 @@
         <v>74</v>
       </c>
       <c r="B75" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="C75" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="D75">
         <v>5</v>
@@ -3210,10 +3228,10 @@
         <v>75</v>
       </c>
       <c r="B76" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="C76" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="D76">
         <v>5</v>
@@ -3227,10 +3245,10 @@
         <v>76</v>
       </c>
       <c r="B77" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C77" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="D77">
         <v>5</v>
@@ -3244,10 +3262,10 @@
         <v>77</v>
       </c>
       <c r="B78" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="C78" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="D78">
         <v>3</v>
@@ -3261,10 +3279,10 @@
         <v>78</v>
       </c>
       <c r="B79" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="C79" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="D79">
         <v>3</v>
@@ -3278,10 +3296,10 @@
         <v>79</v>
       </c>
       <c r="B80" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C80" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="D80">
         <v>3</v>
@@ -3295,10 +3313,10 @@
         <v>80</v>
       </c>
       <c r="B81" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="C81" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="D81">
         <v>9</v>
@@ -3312,10 +3330,10 @@
         <v>81</v>
       </c>
       <c r="B82" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="C82" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="D82">
         <v>9</v>
@@ -3329,10 +3347,10 @@
         <v>82</v>
       </c>
       <c r="B83" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C83" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="D83">
         <v>9</v>
@@ -3346,10 +3364,10 @@
         <v>83</v>
       </c>
       <c r="B84" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="C84" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="D84">
         <v>9</v>
@@ -3363,10 +3381,10 @@
         <v>84</v>
       </c>
       <c r="B85" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="C85" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="D85">
         <v>9</v>
@@ -3380,10 +3398,10 @@
         <v>85</v>
       </c>
       <c r="B86" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="C86" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D86">
         <v>11</v>
@@ -3397,10 +3415,10 @@
         <v>86</v>
       </c>
       <c r="B87" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="C87" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="D87">
         <v>11</v>
@@ -3414,10 +3432,10 @@
         <v>87</v>
       </c>
       <c r="B88" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="C88" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="D88">
         <v>11</v>
@@ -3431,10 +3449,10 @@
         <v>88</v>
       </c>
       <c r="B89" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="C89" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="D89">
         <v>12</v>
@@ -3448,10 +3466,10 @@
         <v>89</v>
       </c>
       <c r="B90" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C90" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="D90">
         <v>12</v>
@@ -3465,10 +3483,10 @@
         <v>90</v>
       </c>
       <c r="B91" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="C91" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="D91">
         <v>12</v>
@@ -3482,10 +3500,10 @@
         <v>91</v>
       </c>
       <c r="B92" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="C92" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="D92">
         <v>14</v>
@@ -3499,10 +3517,10 @@
         <v>92</v>
       </c>
       <c r="B93" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="C93" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="D93">
         <v>14</v>
@@ -3516,10 +3534,10 @@
         <v>93</v>
       </c>
       <c r="B94" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="C94" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="D94">
         <v>13</v>
@@ -3533,10 +3551,10 @@
         <v>94</v>
       </c>
       <c r="B95" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="C95" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="D95">
         <v>13</v>
@@ -3550,10 +3568,10 @@
         <v>95</v>
       </c>
       <c r="B96" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C96" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="D96">
         <v>15</v>
@@ -3567,10 +3585,10 @@
         <v>96</v>
       </c>
       <c r="B97" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C97" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="D97">
         <v>15</v>
@@ -3584,10 +3602,10 @@
         <v>97</v>
       </c>
       <c r="B98" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="C98" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="D98">
         <v>16</v>
@@ -3601,10 +3619,10 @@
         <v>98</v>
       </c>
       <c r="B99" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="C99" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="D99">
         <v>16</v>
@@ -3618,10 +3636,10 @@
         <v>99</v>
       </c>
       <c r="B100" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="C100" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="D100">
         <v>20</v>
@@ -3635,10 +3653,10 @@
         <v>100</v>
       </c>
       <c r="B101" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C101" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="D101">
         <v>20</v>
@@ -3665,16 +3683,16 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="C1" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="D1" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="E1" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -3685,7 +3703,7 @@
         <v>12000</v>
       </c>
       <c r="C2" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="D2">
         <v>150</v>
@@ -3702,7 +3720,7 @@
         <v>13000</v>
       </c>
       <c r="C3" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="D3">
         <v>140</v>
@@ -3719,7 +3737,7 @@
         <v>14000</v>
       </c>
       <c r="C4" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="D4">
         <v>120</v>
@@ -3736,7 +3754,7 @@
         <v>10000</v>
       </c>
       <c r="C5" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="D5">
         <v>300</v>
@@ -3753,7 +3771,7 @@
         <v>10000</v>
       </c>
       <c r="C6" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="D6">
         <v>250</v>
@@ -3770,7 +3788,7 @@
         <v>10000</v>
       </c>
       <c r="C7" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="D7">
         <v>280</v>
@@ -3787,7 +3805,7 @@
         <v>12000</v>
       </c>
       <c r="C8" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="D8">
         <v>180</v>
@@ -3804,7 +3822,7 @@
         <v>15000</v>
       </c>
       <c r="C9" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="D9">
         <v>160</v>
@@ -3821,7 +3839,7 @@
         <v>18000</v>
       </c>
       <c r="C10" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="D10">
         <v>100</v>
@@ -3838,7 +3856,7 @@
         <v>18000</v>
       </c>
       <c r="C11" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="D11">
         <v>100</v>
@@ -3855,7 +3873,7 @@
         <v>35000</v>
       </c>
       <c r="C12" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="D12">
         <v>80</v>
@@ -3872,7 +3890,7 @@
         <v>28000</v>
       </c>
       <c r="C13" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="D13">
         <v>90</v>
@@ -3889,7 +3907,7 @@
         <v>45000</v>
       </c>
       <c r="C14" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="D14">
         <v>60</v>
@@ -3906,7 +3924,7 @@
         <v>5000</v>
       </c>
       <c r="C15" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="D15">
         <v>400</v>
@@ -3923,7 +3941,7 @@
         <v>8000</v>
       </c>
       <c r="C16" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="D16">
         <v>300</v>
@@ -3940,7 +3958,7 @@
         <v>4500</v>
       </c>
       <c r="C17" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="D17">
         <v>350</v>
@@ -3957,7 +3975,7 @@
         <v>9000</v>
       </c>
       <c r="C18" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="D18">
         <v>250</v>
@@ -3974,7 +3992,7 @@
         <v>22000</v>
       </c>
       <c r="C19" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="D19">
         <v>120</v>
@@ -3991,7 +4009,7 @@
         <v>22000</v>
       </c>
       <c r="C20" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="D20">
         <v>120</v>
@@ -4008,7 +4026,7 @@
         <v>55000</v>
       </c>
       <c r="C21" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="D21">
         <v>70</v>
@@ -4025,7 +4043,7 @@
         <v>20000</v>
       </c>
       <c r="C22" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="D22">
         <v>90</v>
@@ -4042,7 +4060,7 @@
         <v>45000</v>
       </c>
       <c r="C23" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="D23">
         <v>150</v>
@@ -4059,7 +4077,7 @@
         <v>22000</v>
       </c>
       <c r="C24" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="D24">
         <v>120</v>
@@ -4076,7 +4094,7 @@
         <v>10000</v>
       </c>
       <c r="C25" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="D25">
         <v>220</v>
@@ -4093,7 +4111,7 @@
         <v>12000</v>
       </c>
       <c r="C26" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="D26">
         <v>150</v>
@@ -4110,7 +4128,7 @@
         <v>12000</v>
       </c>
       <c r="C27" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="D27">
         <v>180</v>
@@ -4127,7 +4145,7 @@
         <v>7000</v>
       </c>
       <c r="C28" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="D28">
         <v>500</v>
@@ -4144,7 +4162,7 @@
         <v>7000</v>
       </c>
       <c r="C29" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="D29">
         <v>500</v>
@@ -4161,7 +4179,7 @@
         <v>5000</v>
       </c>
       <c r="C30" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="D30">
         <v>300</v>
@@ -4178,7 +4196,7 @@
         <v>36000</v>
       </c>
       <c r="C31" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="D31">
         <v>80</v>
@@ -4195,7 +4213,7 @@
         <v>18000</v>
       </c>
       <c r="C32" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="D32">
         <v>140</v>
@@ -4212,7 +4230,7 @@
         <v>12000</v>
       </c>
       <c r="C33" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="D33">
         <v>160</v>
@@ -4229,7 +4247,7 @@
         <v>15000</v>
       </c>
       <c r="C34" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="D34">
         <v>170</v>
@@ -4246,7 +4264,7 @@
         <v>13000</v>
       </c>
       <c r="C35" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="D35">
         <v>120</v>
@@ -4263,7 +4281,7 @@
         <v>15000</v>
       </c>
       <c r="C36" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="D36">
         <v>110</v>
@@ -4280,7 +4298,7 @@
         <v>12000</v>
       </c>
       <c r="C37" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="D37">
         <v>200</v>
@@ -4297,7 +4315,7 @@
         <v>12000</v>
       </c>
       <c r="C38" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="D38">
         <v>180</v>
@@ -4314,7 +4332,7 @@
         <v>16000</v>
       </c>
       <c r="C39" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="D39">
         <v>120</v>
@@ -4331,7 +4349,7 @@
         <v>18000</v>
       </c>
       <c r="C40" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="D40">
         <v>100</v>
@@ -4348,7 +4366,7 @@
         <v>35000</v>
       </c>
       <c r="C41" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="D41">
         <v>80</v>
@@ -4365,7 +4383,7 @@
         <v>6000</v>
       </c>
       <c r="C42" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="D42">
         <v>250</v>
@@ -4382,7 +4400,7 @@
         <v>9000</v>
       </c>
       <c r="C43" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="D43">
         <v>240</v>
@@ -4399,7 +4417,7 @@
         <v>5000</v>
       </c>
       <c r="C44" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="D44">
         <v>260</v>
@@ -4416,7 +4434,7 @@
         <v>10000</v>
       </c>
       <c r="C45" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="D45">
         <v>180</v>
@@ -4433,7 +4451,7 @@
         <v>22000</v>
       </c>
       <c r="C46" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="D46">
         <v>120</v>
@@ -4450,7 +4468,7 @@
         <v>55000</v>
       </c>
       <c r="C47" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="D47">
         <v>70</v>
@@ -4467,7 +4485,7 @@
         <v>18000</v>
       </c>
       <c r="C48" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="D48">
         <v>90</v>
@@ -4484,7 +4502,7 @@
         <v>50000</v>
       </c>
       <c r="C49" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="D49">
         <v>100</v>
@@ -4501,7 +4519,7 @@
         <v>24000</v>
       </c>
       <c r="C50" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="D50">
         <v>110</v>
@@ -4518,7 +4536,7 @@
         <v>10000</v>
       </c>
       <c r="C51" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="D51">
         <v>210</v>
@@ -4535,7 +4553,7 @@
         <v>12000</v>
       </c>
       <c r="C52" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="D52">
         <v>150</v>
@@ -4552,7 +4570,7 @@
         <v>14000</v>
       </c>
       <c r="C53" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="D53">
         <v>130</v>
@@ -4569,7 +4587,7 @@
         <v>9000</v>
       </c>
       <c r="C54" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="D54">
         <v>200</v>
@@ -4586,7 +4604,7 @@
         <v>9000</v>
       </c>
       <c r="C55" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="D55">
         <v>180</v>
@@ -4603,7 +4621,7 @@
         <v>20000</v>
       </c>
       <c r="C56" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="D56">
         <v>100</v>
@@ -4620,7 +4638,7 @@
         <v>12000</v>
       </c>
       <c r="C57" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="D57">
         <v>120</v>
@@ -4637,7 +4655,7 @@
         <v>15000</v>
       </c>
       <c r="C58" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="D58">
         <v>110</v>
@@ -4654,7 +4672,7 @@
         <v>18000</v>
       </c>
       <c r="C59" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="D59">
         <v>50</v>
@@ -4671,7 +4689,7 @@
         <v>22000</v>
       </c>
       <c r="C60" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="D60">
         <v>40</v>
@@ -4688,7 +4706,7 @@
         <v>35000</v>
       </c>
       <c r="C61" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="D61">
         <v>35</v>
@@ -4705,7 +4723,7 @@
         <v>42000</v>
       </c>
       <c r="C62" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="D62">
         <v>30</v>
@@ -4722,7 +4740,7 @@
         <v>42000</v>
       </c>
       <c r="C63" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="D63">
         <v>25</v>
@@ -4739,7 +4757,7 @@
         <v>28000</v>
       </c>
       <c r="C64" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="D64">
         <v>60</v>
@@ -4756,7 +4774,7 @@
         <v>85000</v>
       </c>
       <c r="C65" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="D65">
         <v>20</v>
@@ -4773,7 +4791,7 @@
         <v>45000</v>
       </c>
       <c r="C66" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="D66">
         <v>40</v>
@@ -4790,7 +4808,7 @@
         <v>45000</v>
       </c>
       <c r="C67" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="D67">
         <v>40</v>
@@ -4807,7 +4825,7 @@
         <v>25000</v>
       </c>
       <c r="C68" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="D68">
         <v>50</v>
@@ -4824,7 +4842,7 @@
         <v>30000</v>
       </c>
       <c r="C69" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="D69">
         <v>60</v>
@@ -4841,7 +4859,7 @@
         <v>45000</v>
       </c>
       <c r="C70" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="D70">
         <v>40</v>
@@ -4858,7 +4876,7 @@
         <v>18000</v>
       </c>
       <c r="C71" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="D71">
         <v>45</v>
@@ -4875,7 +4893,7 @@
         <v>95000</v>
       </c>
       <c r="C72" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="D72">
         <v>35</v>
@@ -4892,7 +4910,7 @@
         <v>140000</v>
       </c>
       <c r="C73" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="D73">
         <v>25</v>
@@ -4909,7 +4927,7 @@
         <v>38000</v>
       </c>
       <c r="C74" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="D74">
         <v>80</v>
@@ -4926,7 +4944,7 @@
         <v>25000</v>
       </c>
       <c r="C75" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="D75">
         <v>60</v>
@@ -4943,7 +4961,7 @@
         <v>18000</v>
       </c>
       <c r="C76" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="D76">
         <v>50</v>
@@ -4960,7 +4978,7 @@
         <v>30000</v>
       </c>
       <c r="C77" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="D77">
         <v>35</v>
@@ -4977,7 +4995,7 @@
         <v>22000</v>
       </c>
       <c r="C78" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="D78">
         <v>90</v>
@@ -4994,7 +5012,7 @@
         <v>18000</v>
       </c>
       <c r="C79" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="D79">
         <v>120</v>
@@ -5011,7 +5029,7 @@
         <v>20000</v>
       </c>
       <c r="C80" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="D80">
         <v>100</v>
@@ -5028,7 +5046,7 @@
         <v>42000</v>
       </c>
       <c r="C81" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="D81">
         <v>80</v>
@@ -5045,7 +5063,7 @@
         <v>38000</v>
       </c>
       <c r="C82" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="D82">
         <v>80</v>
@@ -5062,7 +5080,7 @@
         <v>35000</v>
       </c>
       <c r="C83" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="D83">
         <v>60</v>
@@ -5079,7 +5097,7 @@
         <v>28000</v>
       </c>
       <c r="C84" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="D84">
         <v>70</v>
@@ -5096,7 +5114,7 @@
         <v>32000</v>
       </c>
       <c r="C85" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="D85">
         <v>60</v>
@@ -5113,7 +5131,7 @@
         <v>75000</v>
       </c>
       <c r="C86" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="D86">
         <v>40</v>
@@ -5130,7 +5148,7 @@
         <v>85000</v>
       </c>
       <c r="C87" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="D87">
         <v>35</v>
@@ -5147,7 +5165,7 @@
         <v>42000</v>
       </c>
       <c r="C88" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="D88">
         <v>70</v>
@@ -5164,7 +5182,7 @@
         <v>120000</v>
       </c>
       <c r="C89" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="D89">
         <v>30</v>
@@ -5181,7 +5199,7 @@
         <v>38000</v>
       </c>
       <c r="C90" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="D90">
         <v>50</v>
@@ -5198,7 +5216,7 @@
         <v>28000</v>
       </c>
       <c r="C91" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="D91">
         <v>100</v>
@@ -5215,7 +5233,7 @@
         <v>90000</v>
       </c>
       <c r="C92" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="D92">
         <v>20</v>
@@ -5232,7 +5250,7 @@
         <v>150000</v>
       </c>
       <c r="C93" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="D93">
         <v>15</v>
@@ -5249,7 +5267,7 @@
         <v>320000</v>
       </c>
       <c r="C94" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="D94">
         <v>20</v>
@@ -5266,7 +5284,7 @@
         <v>45000</v>
       </c>
       <c r="C95" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="D95">
         <v>50</v>
@@ -5283,7 +5301,7 @@
         <v>35000</v>
       </c>
       <c r="C96" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="D96">
         <v>100</v>
@@ -5300,7 +5318,7 @@
         <v>38000</v>
       </c>
       <c r="C97" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="D97">
         <v>90</v>
@@ -5317,7 +5335,7 @@
         <v>22000</v>
       </c>
       <c r="C98" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="D98">
         <v>150</v>
@@ -5334,7 +5352,7 @@
         <v>28000</v>
       </c>
       <c r="C99" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="D99">
         <v>120</v>
@@ -5351,7 +5369,7 @@
         <v>85000</v>
       </c>
       <c r="C100" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="D100">
         <v>30</v>
@@ -5368,7 +5386,7 @@
         <v>150000</v>
       </c>
       <c r="C101" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="D101">
         <v>20</v>

</xml_diff>

<commit_message>
Restrict setters for Branch properties; update Excel data
Changed Branch entity properties to use private setters for better encapsulation and data integrity. Updated ConvenienceStoreData.xlsx with new data.
</commit_message>
<xml_diff>
--- a/src/External/ConvenienceStore.Persistence/Data/ConvenienceStoreData.xlsx
+++ b/src/External/ConvenienceStore.Persistence/Data/ConvenienceStoreData.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30318"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30327"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="224" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{896CB1D0-8542-4B93-9B07-55FBC7011617}"/>
+  <xr:revisionPtr revIDLastSave="229" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A2DB5C00-1EA0-4EE0-9D89-22352F35D4CE}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Categories" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="665" uniqueCount="347">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="637" uniqueCount="346">
   <si>
     <t>Id</t>
   </si>
@@ -860,9 +860,6 @@
   </si>
   <si>
     <t>Tub</t>
-  </si>
-  <si>
-    <t>Kg</t>
   </si>
   <si>
     <t>Cup</t>
@@ -5670,7 +5667,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B485A97C-E092-4E06-B68C-90ECE5645DB1}">
-  <dimension ref="A1:E99"/>
+  <dimension ref="A1:E71"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="4" max="4" width="16" bestFit="1" customWidth="1"/>
@@ -6800,563 +6797,87 @@
     </row>
     <row r="67" spans="1:5">
       <c r="A67">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="B67">
         <v>25000</v>
       </c>
       <c r="C67" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="D67">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="E67">
-        <v>67</v>
+        <v>74</v>
       </c>
     </row>
     <row r="68" spans="1:5">
       <c r="A68">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="B68">
-        <v>30000</v>
+        <v>18000</v>
       </c>
       <c r="C68" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="D68">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="E68">
-        <v>68</v>
+        <v>75</v>
       </c>
     </row>
     <row r="69" spans="1:5">
       <c r="A69">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="B69">
-        <v>45000</v>
+        <v>22000</v>
       </c>
       <c r="C69" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
       <c r="D69">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="E69">
-        <v>69</v>
+        <v>77</v>
       </c>
     </row>
     <row r="70" spans="1:5">
       <c r="A70">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="B70">
         <v>18000</v>
       </c>
       <c r="C70" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="D70">
-        <v>45</v>
+        <v>120</v>
       </c>
       <c r="E70">
-        <v>70</v>
+        <v>78</v>
       </c>
     </row>
     <row r="71" spans="1:5">
       <c r="A71">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="B71">
-        <v>95000</v>
+        <v>20000</v>
       </c>
       <c r="C71" t="s">
         <v>265</v>
       </c>
       <c r="D71">
-        <v>35</v>
+        <v>100</v>
       </c>
       <c r="E71">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="72" spans="1:5">
-      <c r="A72">
-        <v>72</v>
-      </c>
-      <c r="B72">
-        <v>140000</v>
-      </c>
-      <c r="C72" t="s">
-        <v>265</v>
-      </c>
-      <c r="D72">
-        <v>25</v>
-      </c>
-      <c r="E72">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="73" spans="1:5">
-      <c r="A73">
-        <v>73</v>
-      </c>
-      <c r="B73">
-        <v>38000</v>
-      </c>
-      <c r="C73" t="s">
-        <v>262</v>
-      </c>
-      <c r="D73">
-        <v>80</v>
-      </c>
-      <c r="E73">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="74" spans="1:5">
-      <c r="A74">
-        <v>74</v>
-      </c>
-      <c r="B74">
-        <v>25000</v>
-      </c>
-      <c r="C74" t="s">
-        <v>263</v>
-      </c>
-      <c r="D74">
-        <v>60</v>
-      </c>
-      <c r="E74">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="75" spans="1:5">
-      <c r="A75">
-        <v>75</v>
-      </c>
-      <c r="B75">
-        <v>18000</v>
-      </c>
-      <c r="C75" t="s">
-        <v>263</v>
-      </c>
-      <c r="D75">
-        <v>50</v>
-      </c>
-      <c r="E75">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="76" spans="1:5">
-      <c r="A76">
-        <v>77</v>
-      </c>
-      <c r="B76">
-        <v>22000</v>
-      </c>
-      <c r="C76" t="s">
-        <v>259</v>
-      </c>
-      <c r="D76">
-        <v>90</v>
-      </c>
-      <c r="E76">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="77" spans="1:5">
-      <c r="A77">
-        <v>78</v>
-      </c>
-      <c r="B77">
-        <v>18000</v>
-      </c>
-      <c r="C77" t="s">
-        <v>266</v>
-      </c>
-      <c r="D77">
-        <v>120</v>
-      </c>
-      <c r="E77">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="78" spans="1:5">
-      <c r="A78">
         <v>79</v>
-      </c>
-      <c r="B78">
-        <v>20000</v>
-      </c>
-      <c r="C78" t="s">
-        <v>266</v>
-      </c>
-      <c r="D78">
-        <v>100</v>
-      </c>
-      <c r="E78">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="79" spans="1:5">
-      <c r="A79">
-        <v>80</v>
-      </c>
-      <c r="B79">
-        <v>42000</v>
-      </c>
-      <c r="C79" t="s">
-        <v>260</v>
-      </c>
-      <c r="D79">
-        <v>80</v>
-      </c>
-      <c r="E79">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="80" spans="1:5">
-      <c r="A80">
-        <v>81</v>
-      </c>
-      <c r="B80">
-        <v>38000</v>
-      </c>
-      <c r="C80" t="s">
-        <v>260</v>
-      </c>
-      <c r="D80">
-        <v>80</v>
-      </c>
-      <c r="E80">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="81" spans="1:5">
-      <c r="A81">
-        <v>82</v>
-      </c>
-      <c r="B81">
-        <v>35000</v>
-      </c>
-      <c r="C81" t="s">
-        <v>260</v>
-      </c>
-      <c r="D81">
-        <v>60</v>
-      </c>
-      <c r="E81">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="82" spans="1:5">
-      <c r="A82">
-        <v>83</v>
-      </c>
-      <c r="B82">
-        <v>28000</v>
-      </c>
-      <c r="C82" t="s">
-        <v>258</v>
-      </c>
-      <c r="D82">
-        <v>70</v>
-      </c>
-      <c r="E82">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="83" spans="1:5">
-      <c r="A83">
-        <v>84</v>
-      </c>
-      <c r="B83">
-        <v>32000</v>
-      </c>
-      <c r="C83" t="s">
-        <v>258</v>
-      </c>
-      <c r="D83">
-        <v>60</v>
-      </c>
-      <c r="E83">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="84" spans="1:5">
-      <c r="A84">
-        <v>85</v>
-      </c>
-      <c r="B84">
-        <v>75000</v>
-      </c>
-      <c r="C84" t="s">
-        <v>258</v>
-      </c>
-      <c r="D84">
-        <v>40</v>
-      </c>
-      <c r="E84">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="85" spans="1:5">
-      <c r="A85">
-        <v>86</v>
-      </c>
-      <c r="B85">
-        <v>85000</v>
-      </c>
-      <c r="C85" t="s">
-        <v>258</v>
-      </c>
-      <c r="D85">
-        <v>35</v>
-      </c>
-      <c r="E85">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="86" spans="1:5">
-      <c r="A86">
-        <v>87</v>
-      </c>
-      <c r="B86">
-        <v>42000</v>
-      </c>
-      <c r="C86" t="s">
-        <v>259</v>
-      </c>
-      <c r="D86">
-        <v>70</v>
-      </c>
-      <c r="E86">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="87" spans="1:5">
-      <c r="A87">
-        <v>88</v>
-      </c>
-      <c r="B87">
-        <v>120000</v>
-      </c>
-      <c r="C87" t="s">
-        <v>258</v>
-      </c>
-      <c r="D87">
-        <v>30</v>
-      </c>
-      <c r="E87">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="88" spans="1:5">
-      <c r="A88">
-        <v>89</v>
-      </c>
-      <c r="B88">
-        <v>38000</v>
-      </c>
-      <c r="C88" t="s">
-        <v>258</v>
-      </c>
-      <c r="D88">
-        <v>50</v>
-      </c>
-      <c r="E88">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="89" spans="1:5">
-      <c r="A89">
-        <v>90</v>
-      </c>
-      <c r="B89">
-        <v>28000</v>
-      </c>
-      <c r="C89" t="s">
-        <v>259</v>
-      </c>
-      <c r="D89">
-        <v>100</v>
-      </c>
-      <c r="E89">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="90" spans="1:5">
-      <c r="A90">
-        <v>91</v>
-      </c>
-      <c r="B90">
-        <v>90000</v>
-      </c>
-      <c r="C90" t="s">
-        <v>261</v>
-      </c>
-      <c r="D90">
-        <v>20</v>
-      </c>
-      <c r="E90">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="91" spans="1:5">
-      <c r="A91">
-        <v>92</v>
-      </c>
-      <c r="B91">
-        <v>150000</v>
-      </c>
-      <c r="C91" t="s">
-        <v>261</v>
-      </c>
-      <c r="D91">
-        <v>15</v>
-      </c>
-      <c r="E91">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="92" spans="1:5">
-      <c r="A92">
-        <v>93</v>
-      </c>
-      <c r="B92">
-        <v>320000</v>
-      </c>
-      <c r="C92" t="s">
-        <v>262</v>
-      </c>
-      <c r="D92">
-        <v>20</v>
-      </c>
-      <c r="E92">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="93" spans="1:5">
-      <c r="A93">
-        <v>94</v>
-      </c>
-      <c r="B93">
-        <v>45000</v>
-      </c>
-      <c r="C93" t="s">
-        <v>262</v>
-      </c>
-      <c r="D93">
-        <v>50</v>
-      </c>
-      <c r="E93">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="94" spans="1:5">
-      <c r="A94">
-        <v>95</v>
-      </c>
-      <c r="B94">
-        <v>35000</v>
-      </c>
-      <c r="C94" t="s">
-        <v>262</v>
-      </c>
-      <c r="D94">
-        <v>100</v>
-      </c>
-      <c r="E94">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="95" spans="1:5">
-      <c r="A95">
-        <v>96</v>
-      </c>
-      <c r="B95">
-        <v>38000</v>
-      </c>
-      <c r="C95" t="s">
-        <v>262</v>
-      </c>
-      <c r="D95">
-        <v>90</v>
-      </c>
-      <c r="E95">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="96" spans="1:5">
-      <c r="A96">
-        <v>97</v>
-      </c>
-      <c r="B96">
-        <v>22000</v>
-      </c>
-      <c r="C96" t="s">
-        <v>260</v>
-      </c>
-      <c r="D96">
-        <v>150</v>
-      </c>
-      <c r="E96">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="97" spans="1:5">
-      <c r="A97">
-        <v>98</v>
-      </c>
-      <c r="B97">
-        <v>28000</v>
-      </c>
-      <c r="C97" t="s">
-        <v>258</v>
-      </c>
-      <c r="D97">
-        <v>120</v>
-      </c>
-      <c r="E97">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="98" spans="1:5">
-      <c r="A98">
-        <v>99</v>
-      </c>
-      <c r="B98">
-        <v>85000</v>
-      </c>
-      <c r="C98" t="s">
-        <v>259</v>
-      </c>
-      <c r="D98">
-        <v>30</v>
-      </c>
-      <c r="E98">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="99" spans="1:5">
-      <c r="A99">
-        <v>100</v>
-      </c>
-      <c r="B99">
-        <v>150000</v>
-      </c>
-      <c r="C99" t="s">
-        <v>259</v>
-      </c>
-      <c r="D99">
-        <v>20</v>
-      </c>
-      <c r="E99">
-        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -7388,10 +6909,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>266</v>
+      </c>
+      <c r="C2" t="s">
         <v>267</v>
-      </c>
-      <c r="C2" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -7399,10 +6920,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
+        <v>268</v>
+      </c>
+      <c r="C3" t="s">
         <v>269</v>
-      </c>
-      <c r="C3" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -7410,10 +6931,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
+        <v>270</v>
+      </c>
+      <c r="C4" t="s">
         <v>271</v>
-      </c>
-      <c r="C4" t="s">
-        <v>272</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -7421,10 +6942,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
+        <v>272</v>
+      </c>
+      <c r="C5" t="s">
         <v>273</v>
-      </c>
-      <c r="C5" t="s">
-        <v>274</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -7432,10 +6953,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
+        <v>274</v>
+      </c>
+      <c r="C6" t="s">
         <v>275</v>
-      </c>
-      <c r="C6" t="s">
-        <v>276</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -7443,10 +6964,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C7" t="s">
         <v>277</v>
-      </c>
-      <c r="C7" t="s">
-        <v>278</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -7454,10 +6975,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
+        <v>278</v>
+      </c>
+      <c r="C8" t="s">
         <v>279</v>
-      </c>
-      <c r="C8" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -7465,10 +6986,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
+        <v>280</v>
+      </c>
+      <c r="C9" t="s">
         <v>281</v>
-      </c>
-      <c r="C9" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -7476,10 +6997,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
+        <v>282</v>
+      </c>
+      <c r="C10" t="s">
         <v>283</v>
-      </c>
-      <c r="C10" t="s">
-        <v>284</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -7487,10 +7008,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
+        <v>284</v>
+      </c>
+      <c r="C11" t="s">
         <v>285</v>
-      </c>
-      <c r="C11" t="s">
-        <v>286</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -7498,10 +7019,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
+        <v>286</v>
+      </c>
+      <c r="C12" t="s">
         <v>287</v>
-      </c>
-      <c r="C12" t="s">
-        <v>288</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -7509,10 +7030,10 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
+        <v>288</v>
+      </c>
+      <c r="C13" t="s">
         <v>289</v>
-      </c>
-      <c r="C13" t="s">
-        <v>290</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -7520,10 +7041,10 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
+        <v>290</v>
+      </c>
+      <c r="C14" t="s">
         <v>291</v>
-      </c>
-      <c r="C14" t="s">
-        <v>292</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -7531,10 +7052,10 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
+        <v>292</v>
+      </c>
+      <c r="C15" t="s">
         <v>293</v>
-      </c>
-      <c r="C15" t="s">
-        <v>294</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -7542,10 +7063,10 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
+        <v>294</v>
+      </c>
+      <c r="C16" t="s">
         <v>295</v>
-      </c>
-      <c r="C16" t="s">
-        <v>296</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -7553,10 +7074,10 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
+        <v>296</v>
+      </c>
+      <c r="C17" t="s">
         <v>297</v>
-      </c>
-      <c r="C17" t="s">
-        <v>298</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -7564,10 +7085,10 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
+        <v>298</v>
+      </c>
+      <c r="C18" t="s">
         <v>299</v>
-      </c>
-      <c r="C18" t="s">
-        <v>300</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -7575,10 +7096,10 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
+        <v>300</v>
+      </c>
+      <c r="C19" t="s">
         <v>301</v>
-      </c>
-      <c r="C19" t="s">
-        <v>302</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -7586,10 +7107,10 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
+        <v>302</v>
+      </c>
+      <c r="C20" t="s">
         <v>303</v>
-      </c>
-      <c r="C20" t="s">
-        <v>304</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -7597,10 +7118,10 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
+        <v>304</v>
+      </c>
+      <c r="C21" t="s">
         <v>305</v>
-      </c>
-      <c r="C21" t="s">
-        <v>306</v>
       </c>
     </row>
     <row r="22" spans="1:3">
@@ -7608,10 +7129,10 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
+        <v>306</v>
+      </c>
+      <c r="C22" t="s">
         <v>307</v>
-      </c>
-      <c r="C22" t="s">
-        <v>308</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -7619,10 +7140,10 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
+        <v>308</v>
+      </c>
+      <c r="C23" t="s">
         <v>309</v>
-      </c>
-      <c r="C23" t="s">
-        <v>310</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -7630,10 +7151,10 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
+        <v>310</v>
+      </c>
+      <c r="C24" t="s">
         <v>311</v>
-      </c>
-      <c r="C24" t="s">
-        <v>312</v>
       </c>
     </row>
     <row r="25" spans="1:3">
@@ -7641,10 +7162,10 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
+        <v>312</v>
+      </c>
+      <c r="C25" t="s">
         <v>313</v>
-      </c>
-      <c r="C25" t="s">
-        <v>314</v>
       </c>
     </row>
     <row r="26" spans="1:3">
@@ -7652,10 +7173,10 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
+        <v>314</v>
+      </c>
+      <c r="C26" t="s">
         <v>315</v>
-      </c>
-      <c r="C26" t="s">
-        <v>316</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -7663,10 +7184,10 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
+        <v>316</v>
+      </c>
+      <c r="C27" t="s">
         <v>317</v>
-      </c>
-      <c r="C27" t="s">
-        <v>318</v>
       </c>
     </row>
     <row r="28" spans="1:3">
@@ -7674,10 +7195,10 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
+        <v>318</v>
+      </c>
+      <c r="C28" t="s">
         <v>319</v>
-      </c>
-      <c r="C28" t="s">
-        <v>320</v>
       </c>
     </row>
     <row r="29" spans="1:3">
@@ -7685,10 +7206,10 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
+        <v>320</v>
+      </c>
+      <c r="C29" t="s">
         <v>321</v>
-      </c>
-      <c r="C29" t="s">
-        <v>322</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -7696,10 +7217,10 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
+        <v>322</v>
+      </c>
+      <c r="C30" t="s">
         <v>323</v>
-      </c>
-      <c r="C30" t="s">
-        <v>324</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -7707,10 +7228,10 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
+        <v>324</v>
+      </c>
+      <c r="C31" t="s">
         <v>325</v>
-      </c>
-      <c r="C31" t="s">
-        <v>326</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -7718,10 +7239,10 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
+        <v>326</v>
+      </c>
+      <c r="C32" t="s">
         <v>327</v>
-      </c>
-      <c r="C32" t="s">
-        <v>328</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -7729,10 +7250,10 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
+        <v>328</v>
+      </c>
+      <c r="C33" t="s">
         <v>329</v>
-      </c>
-      <c r="C33" t="s">
-        <v>330</v>
       </c>
     </row>
     <row r="34" spans="1:3">
@@ -7740,10 +7261,10 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
+        <v>330</v>
+      </c>
+      <c r="C34" t="s">
         <v>331</v>
-      </c>
-      <c r="C34" t="s">
-        <v>332</v>
       </c>
     </row>
     <row r="35" spans="1:3">
@@ -7751,7 +7272,7 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="36" spans="1:3">
@@ -7759,10 +7280,10 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
+        <v>333</v>
+      </c>
+      <c r="C36" t="s">
         <v>334</v>
-      </c>
-      <c r="C36" t="s">
-        <v>335</v>
       </c>
     </row>
     <row r="37" spans="1:3">
@@ -7770,10 +7291,10 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
+        <v>335</v>
+      </c>
+      <c r="C37" t="s">
         <v>336</v>
-      </c>
-      <c r="C37" t="s">
-        <v>337</v>
       </c>
     </row>
     <row r="38" spans="1:3">
@@ -7781,10 +7302,10 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
+        <v>337</v>
+      </c>
+      <c r="C38" t="s">
         <v>338</v>
-      </c>
-      <c r="C38" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="39" spans="1:3">
@@ -7792,10 +7313,10 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
+        <v>339</v>
+      </c>
+      <c r="C39" t="s">
         <v>340</v>
-      </c>
-      <c r="C39" t="s">
-        <v>341</v>
       </c>
     </row>
     <row r="40" spans="1:3">
@@ -7803,7 +7324,7 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
     <row r="41" spans="1:3">
@@ -7811,10 +7332,10 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
+        <v>342</v>
+      </c>
+      <c r="C41" t="s">
         <v>343</v>
-      </c>
-      <c r="C41" t="s">
-        <v>344</v>
       </c>
     </row>
     <row r="42" spans="1:3">
@@ -7822,10 +7343,10 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
+        <v>344</v>
+      </c>
+      <c r="C42" t="s">
         <v>345</v>
-      </c>
-      <c r="C42" t="s">
-        <v>346</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refactor: move UnitPrice from ProductStock to ProductPrice
Separated product pricing into a new ProductPrice entity. Updated all references, mappings, and configurations to use ProductPrice instead of ProductStock for pricing. Adjusted seeders and data files accordingly for improved separation of concerns.
</commit_message>
<xml_diff>
--- a/src/External/ConvenienceStore.Persistence/Data/ConvenienceStoreData.xlsx
+++ b/src/External/ConvenienceStore.Persistence/Data/ConvenienceStoreData.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30327"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="229" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A2DB5C00-1EA0-4EE0-9D89-22352F35D4CE}"/>
+  <xr:revisionPtr revIDLastSave="239" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6A7B0C29-07F3-4D4E-A61B-1D522CD334A4}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="4" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Categories" sheetId="1" r:id="rId1"/>
@@ -13,7 +13,8 @@
     <sheet name="ProductImages" sheetId="6" r:id="rId3"/>
     <sheet name="Products" sheetId="3" r:id="rId4"/>
     <sheet name="ProductStocks" sheetId="4" r:id="rId5"/>
-    <sheet name="Brands" sheetId="2" r:id="rId6"/>
+    <sheet name="ProductPrices" sheetId="7" r:id="rId6"/>
+    <sheet name="Brands" sheetId="2" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="637" uniqueCount="346">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="639" uniqueCount="346">
   <si>
     <t>Id</t>
   </si>
@@ -832,37 +833,37 @@
     <t>Cup noodles</t>
   </si>
   <si>
+    <t>Unit</t>
+  </si>
+  <si>
+    <t>QuantityOnHand</t>
+  </si>
+  <si>
+    <t>Bottle</t>
+  </si>
+  <si>
+    <t>Box</t>
+  </si>
+  <si>
+    <t>Can</t>
+  </si>
+  <si>
+    <t>Bag</t>
+  </si>
+  <si>
+    <t>Pack</t>
+  </si>
+  <si>
+    <t>Piece</t>
+  </si>
+  <si>
+    <t>Tub</t>
+  </si>
+  <si>
+    <t>Cup</t>
+  </si>
+  <si>
     <t>UnitPrice</t>
-  </si>
-  <si>
-    <t>Unit</t>
-  </si>
-  <si>
-    <t>QuantityOnHand</t>
-  </si>
-  <si>
-    <t>Bottle</t>
-  </si>
-  <si>
-    <t>Box</t>
-  </si>
-  <si>
-    <t>Can</t>
-  </si>
-  <si>
-    <t>Bag</t>
-  </si>
-  <si>
-    <t>Pack</t>
-  </si>
-  <si>
-    <t>Piece</t>
-  </si>
-  <si>
-    <t>Tub</t>
-  </si>
-  <si>
-    <t>Cup</t>
   </si>
   <si>
     <t>Vinamilk</t>
@@ -5667,13 +5668,13 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B485A97C-E092-4E06-B68C-90ECE5645DB1}">
-  <dimension ref="A1:E71"/>
+  <dimension ref="A1:D71"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="4" max="4" width="16" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -5684,1199 +5685,986 @@
         <v>256</v>
       </c>
       <c r="D1" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
         <v>257</v>
       </c>
-      <c r="E1" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>12000</v>
-      </c>
-      <c r="C2" t="s">
-        <v>258</v>
+      <c r="C2">
+        <v>150</v>
       </c>
       <c r="D2">
-        <v>150</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3">
-        <v>13000</v>
-      </c>
-      <c r="C3" t="s">
-        <v>258</v>
+      <c r="B3" t="s">
+        <v>257</v>
+      </c>
+      <c r="C3">
+        <v>140</v>
       </c>
       <c r="D3">
-        <v>140</v>
-      </c>
-      <c r="E3">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:4">
       <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4">
-        <v>14000</v>
-      </c>
-      <c r="C4" t="s">
-        <v>259</v>
+      <c r="B4" t="s">
+        <v>258</v>
+      </c>
+      <c r="C4">
+        <v>120</v>
       </c>
       <c r="D4">
-        <v>120</v>
-      </c>
-      <c r="E4">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:4">
       <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5">
-        <v>10000</v>
-      </c>
-      <c r="C5" t="s">
-        <v>260</v>
+      <c r="B5" t="s">
+        <v>259</v>
+      </c>
+      <c r="C5">
+        <v>300</v>
       </c>
       <c r="D5">
-        <v>300</v>
-      </c>
-      <c r="E5">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:4">
       <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6">
-        <v>10000</v>
-      </c>
-      <c r="C6" t="s">
-        <v>260</v>
+      <c r="B6" t="s">
+        <v>259</v>
+      </c>
+      <c r="C6">
+        <v>250</v>
       </c>
       <c r="D6">
-        <v>250</v>
-      </c>
-      <c r="E6">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:4">
       <c r="A7">
         <v>6</v>
       </c>
-      <c r="B7">
-        <v>10000</v>
-      </c>
-      <c r="C7" t="s">
-        <v>260</v>
+      <c r="B7" t="s">
+        <v>259</v>
+      </c>
+      <c r="C7">
+        <v>280</v>
       </c>
       <c r="D7">
-        <v>280</v>
-      </c>
-      <c r="E7">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:4">
       <c r="A8">
         <v>7</v>
       </c>
-      <c r="B8">
-        <v>12000</v>
-      </c>
-      <c r="C8" t="s">
-        <v>260</v>
+      <c r="B8" t="s">
+        <v>259</v>
+      </c>
+      <c r="C8">
+        <v>180</v>
       </c>
       <c r="D8">
-        <v>180</v>
-      </c>
-      <c r="E8">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:4">
       <c r="A9">
         <v>8</v>
       </c>
-      <c r="B9">
-        <v>15000</v>
-      </c>
-      <c r="C9" t="s">
-        <v>260</v>
+      <c r="B9" t="s">
+        <v>259</v>
+      </c>
+      <c r="C9">
+        <v>160</v>
       </c>
       <c r="D9">
-        <v>160</v>
-      </c>
-      <c r="E9">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:4">
       <c r="A10">
         <v>9</v>
       </c>
-      <c r="B10">
-        <v>18000</v>
-      </c>
-      <c r="C10" t="s">
-        <v>261</v>
+      <c r="B10" t="s">
+        <v>260</v>
+      </c>
+      <c r="C10">
+        <v>100</v>
       </c>
       <c r="D10">
-        <v>100</v>
-      </c>
-      <c r="E10">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:4">
       <c r="A11">
         <v>10</v>
       </c>
-      <c r="B11">
-        <v>18000</v>
-      </c>
-      <c r="C11" t="s">
-        <v>261</v>
+      <c r="B11" t="s">
+        <v>260</v>
+      </c>
+      <c r="C11">
+        <v>100</v>
       </c>
       <c r="D11">
-        <v>100</v>
-      </c>
-      <c r="E11">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
+    <row r="12" spans="1:4">
       <c r="A12">
         <v>11</v>
       </c>
-      <c r="B12">
-        <v>35000</v>
-      </c>
-      <c r="C12" t="s">
-        <v>259</v>
+      <c r="B12" t="s">
+        <v>258</v>
+      </c>
+      <c r="C12">
+        <v>80</v>
       </c>
       <c r="D12">
-        <v>80</v>
-      </c>
-      <c r="E12">
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" spans="1:4">
       <c r="A13">
         <v>12</v>
       </c>
-      <c r="B13">
-        <v>28000</v>
-      </c>
-      <c r="C13" t="s">
-        <v>259</v>
+      <c r="B13" t="s">
+        <v>258</v>
+      </c>
+      <c r="C13">
+        <v>90</v>
       </c>
       <c r="D13">
-        <v>90</v>
-      </c>
-      <c r="E13">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:5">
+    <row r="14" spans="1:4">
       <c r="A14">
         <v>13</v>
       </c>
-      <c r="B14">
-        <v>45000</v>
-      </c>
-      <c r="C14" t="s">
-        <v>259</v>
+      <c r="B14" t="s">
+        <v>258</v>
+      </c>
+      <c r="C14">
+        <v>60</v>
       </c>
       <c r="D14">
-        <v>60</v>
-      </c>
-      <c r="E14">
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:5">
+    <row r="15" spans="1:4">
       <c r="A15">
         <v>14</v>
       </c>
-      <c r="B15">
-        <v>5000</v>
-      </c>
-      <c r="C15" t="s">
-        <v>262</v>
+      <c r="B15" t="s">
+        <v>261</v>
+      </c>
+      <c r="C15">
+        <v>400</v>
       </c>
       <c r="D15">
-        <v>400</v>
-      </c>
-      <c r="E15">
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:5">
+    <row r="16" spans="1:4">
       <c r="A16">
         <v>15</v>
       </c>
-      <c r="B16">
-        <v>8000</v>
-      </c>
-      <c r="C16" t="s">
-        <v>262</v>
+      <c r="B16" t="s">
+        <v>261</v>
+      </c>
+      <c r="C16">
+        <v>300</v>
       </c>
       <c r="D16">
-        <v>300</v>
-      </c>
-      <c r="E16">
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:5">
+    <row r="17" spans="1:4">
       <c r="A17">
         <v>16</v>
       </c>
-      <c r="B17">
-        <v>4500</v>
-      </c>
-      <c r="C17" t="s">
-        <v>262</v>
+      <c r="B17" t="s">
+        <v>261</v>
+      </c>
+      <c r="C17">
+        <v>350</v>
       </c>
       <c r="D17">
-        <v>350</v>
-      </c>
-      <c r="E17">
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:5">
+    <row r="18" spans="1:4">
       <c r="A18">
         <v>17</v>
       </c>
-      <c r="B18">
-        <v>9000</v>
-      </c>
-      <c r="C18" t="s">
-        <v>262</v>
+      <c r="B18" t="s">
+        <v>261</v>
+      </c>
+      <c r="C18">
+        <v>250</v>
       </c>
       <c r="D18">
-        <v>250</v>
-      </c>
-      <c r="E18">
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:5">
+    <row r="19" spans="1:4">
       <c r="A19">
         <v>18</v>
       </c>
-      <c r="B19">
-        <v>22000</v>
-      </c>
-      <c r="C19" t="s">
-        <v>261</v>
+      <c r="B19" t="s">
+        <v>260</v>
+      </c>
+      <c r="C19">
+        <v>120</v>
       </c>
       <c r="D19">
-        <v>120</v>
-      </c>
-      <c r="E19">
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
+    <row r="20" spans="1:4">
       <c r="A20">
         <v>19</v>
       </c>
-      <c r="B20">
-        <v>22000</v>
-      </c>
-      <c r="C20" t="s">
-        <v>261</v>
+      <c r="B20" t="s">
+        <v>260</v>
+      </c>
+      <c r="C20">
+        <v>120</v>
       </c>
       <c r="D20">
-        <v>120</v>
-      </c>
-      <c r="E20">
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:5">
+    <row r="21" spans="1:4">
       <c r="A21">
         <v>20</v>
       </c>
-      <c r="B21">
-        <v>55000</v>
-      </c>
-      <c r="C21" t="s">
-        <v>260</v>
+      <c r="B21" t="s">
+        <v>259</v>
+      </c>
+      <c r="C21">
+        <v>70</v>
       </c>
       <c r="D21">
-        <v>70</v>
-      </c>
-      <c r="E21">
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:5">
+    <row r="22" spans="1:4">
       <c r="A22">
         <v>21</v>
       </c>
-      <c r="B22">
-        <v>20000</v>
-      </c>
-      <c r="C22" t="s">
-        <v>261</v>
+      <c r="B22" t="s">
+        <v>260</v>
+      </c>
+      <c r="C22">
+        <v>90</v>
       </c>
       <c r="D22">
-        <v>90</v>
-      </c>
-      <c r="E22">
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:5">
+    <row r="23" spans="1:4">
       <c r="A23">
         <v>22</v>
       </c>
-      <c r="B23">
-        <v>45000</v>
-      </c>
-      <c r="C23" t="s">
-        <v>259</v>
+      <c r="B23" t="s">
+        <v>258</v>
+      </c>
+      <c r="C23">
+        <v>150</v>
       </c>
       <c r="D23">
-        <v>150</v>
-      </c>
-      <c r="E23">
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:5">
+    <row r="24" spans="1:4">
       <c r="A24">
         <v>23</v>
       </c>
-      <c r="B24">
-        <v>22000</v>
-      </c>
-      <c r="C24" t="s">
-        <v>260</v>
+      <c r="B24" t="s">
+        <v>259</v>
+      </c>
+      <c r="C24">
+        <v>120</v>
       </c>
       <c r="D24">
-        <v>120</v>
-      </c>
-      <c r="E24">
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:5">
+    <row r="25" spans="1:4">
       <c r="A25">
         <v>24</v>
       </c>
-      <c r="B25">
-        <v>10000</v>
-      </c>
-      <c r="C25" t="s">
-        <v>258</v>
+      <c r="B25" t="s">
+        <v>257</v>
+      </c>
+      <c r="C25">
+        <v>220</v>
       </c>
       <c r="D25">
-        <v>220</v>
-      </c>
-      <c r="E25">
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:5">
+    <row r="26" spans="1:4">
       <c r="A26">
         <v>25</v>
       </c>
-      <c r="B26">
-        <v>12000</v>
-      </c>
-      <c r="C26" t="s">
-        <v>260</v>
+      <c r="B26" t="s">
+        <v>259</v>
+      </c>
+      <c r="C26">
+        <v>150</v>
       </c>
       <c r="D26">
-        <v>150</v>
-      </c>
-      <c r="E26">
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:5">
+    <row r="27" spans="1:4">
       <c r="A27">
         <v>26</v>
       </c>
-      <c r="B27">
-        <v>12000</v>
-      </c>
-      <c r="C27" t="s">
-        <v>260</v>
+      <c r="B27" t="s">
+        <v>259</v>
+      </c>
+      <c r="C27">
+        <v>180</v>
       </c>
       <c r="D27">
-        <v>180</v>
-      </c>
-      <c r="E27">
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:5">
+    <row r="28" spans="1:4">
       <c r="A28">
         <v>27</v>
       </c>
-      <c r="B28">
-        <v>7000</v>
-      </c>
-      <c r="C28" t="s">
-        <v>258</v>
+      <c r="B28" t="s">
+        <v>257</v>
+      </c>
+      <c r="C28">
+        <v>500</v>
       </c>
       <c r="D28">
-        <v>500</v>
-      </c>
-      <c r="E28">
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:5">
+    <row r="29" spans="1:4">
       <c r="A29">
         <v>28</v>
       </c>
-      <c r="B29">
-        <v>7000</v>
-      </c>
-      <c r="C29" t="s">
-        <v>258</v>
+      <c r="B29" t="s">
+        <v>257</v>
+      </c>
+      <c r="C29">
+        <v>500</v>
       </c>
       <c r="D29">
-        <v>500</v>
-      </c>
-      <c r="E29">
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="1:5">
+    <row r="30" spans="1:4">
       <c r="A30">
         <v>29</v>
       </c>
-      <c r="B30">
-        <v>5000</v>
-      </c>
-      <c r="C30" t="s">
-        <v>262</v>
+      <c r="B30" t="s">
+        <v>261</v>
+      </c>
+      <c r="C30">
+        <v>300</v>
       </c>
       <c r="D30">
-        <v>300</v>
-      </c>
-      <c r="E30">
         <v>29</v>
       </c>
     </row>
-    <row r="31" spans="1:5">
+    <row r="31" spans="1:4">
       <c r="A31">
         <v>30</v>
       </c>
-      <c r="B31">
-        <v>36000</v>
-      </c>
-      <c r="C31" t="s">
-        <v>259</v>
+      <c r="B31" t="s">
+        <v>258</v>
+      </c>
+      <c r="C31">
+        <v>80</v>
       </c>
       <c r="D31">
-        <v>80</v>
-      </c>
-      <c r="E31">
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="1:5">
+    <row r="32" spans="1:4">
       <c r="A32">
         <v>31</v>
       </c>
-      <c r="B32">
-        <v>18000</v>
-      </c>
-      <c r="C32" t="s">
-        <v>262</v>
+      <c r="B32" t="s">
+        <v>261</v>
+      </c>
+      <c r="C32">
+        <v>140</v>
       </c>
       <c r="D32">
-        <v>140</v>
-      </c>
-      <c r="E32">
         <v>31</v>
       </c>
     </row>
-    <row r="33" spans="1:5">
+    <row r="33" spans="1:4">
       <c r="A33">
         <v>32</v>
       </c>
-      <c r="B33">
-        <v>12000</v>
-      </c>
-      <c r="C33" t="s">
-        <v>262</v>
+      <c r="B33" t="s">
+        <v>261</v>
+      </c>
+      <c r="C33">
+        <v>160</v>
       </c>
       <c r="D33">
-        <v>160</v>
-      </c>
-      <c r="E33">
         <v>32</v>
       </c>
     </row>
-    <row r="34" spans="1:5">
+    <row r="34" spans="1:4">
       <c r="A34">
         <v>33</v>
       </c>
-      <c r="B34">
-        <v>15000</v>
-      </c>
-      <c r="C34" t="s">
-        <v>262</v>
+      <c r="B34" t="s">
+        <v>261</v>
+      </c>
+      <c r="C34">
+        <v>170</v>
       </c>
       <c r="D34">
-        <v>170</v>
-      </c>
-      <c r="E34">
         <v>33</v>
       </c>
     </row>
-    <row r="35" spans="1:5">
+    <row r="35" spans="1:4">
       <c r="A35">
         <v>34</v>
       </c>
-      <c r="B35">
-        <v>13000</v>
-      </c>
-      <c r="C35" t="s">
-        <v>258</v>
+      <c r="B35" t="s">
+        <v>257</v>
+      </c>
+      <c r="C35">
+        <v>120</v>
       </c>
       <c r="D35">
-        <v>120</v>
-      </c>
-      <c r="E35">
         <v>34</v>
       </c>
     </row>
-    <row r="36" spans="1:5">
+    <row r="36" spans="1:4">
       <c r="A36">
         <v>35</v>
       </c>
-      <c r="B36">
-        <v>15000</v>
-      </c>
-      <c r="C36" t="s">
-        <v>259</v>
+      <c r="B36" t="s">
+        <v>258</v>
+      </c>
+      <c r="C36">
+        <v>110</v>
       </c>
       <c r="D36">
-        <v>110</v>
-      </c>
-      <c r="E36">
         <v>35</v>
       </c>
     </row>
-    <row r="37" spans="1:5">
+    <row r="37" spans="1:4">
       <c r="A37">
         <v>36</v>
       </c>
-      <c r="B37">
-        <v>12000</v>
-      </c>
-      <c r="C37" t="s">
-        <v>260</v>
+      <c r="B37" t="s">
+        <v>259</v>
+      </c>
+      <c r="C37">
+        <v>200</v>
       </c>
       <c r="D37">
-        <v>200</v>
-      </c>
-      <c r="E37">
         <v>36</v>
       </c>
     </row>
-    <row r="38" spans="1:5">
+    <row r="38" spans="1:4">
       <c r="A38">
         <v>37</v>
       </c>
-      <c r="B38">
-        <v>12000</v>
-      </c>
-      <c r="C38" t="s">
-        <v>260</v>
+      <c r="B38" t="s">
+        <v>259</v>
+      </c>
+      <c r="C38">
+        <v>180</v>
       </c>
       <c r="D38">
-        <v>180</v>
-      </c>
-      <c r="E38">
         <v>37</v>
       </c>
     </row>
-    <row r="39" spans="1:5">
+    <row r="39" spans="1:4">
       <c r="A39">
         <v>38</v>
       </c>
-      <c r="B39">
-        <v>16000</v>
-      </c>
-      <c r="C39" t="s">
-        <v>260</v>
+      <c r="B39" t="s">
+        <v>259</v>
+      </c>
+      <c r="C39">
+        <v>120</v>
       </c>
       <c r="D39">
-        <v>120</v>
-      </c>
-      <c r="E39">
         <v>38</v>
       </c>
     </row>
-    <row r="40" spans="1:5">
+    <row r="40" spans="1:4">
       <c r="A40">
         <v>39</v>
       </c>
-      <c r="B40">
-        <v>18000</v>
-      </c>
-      <c r="C40" t="s">
-        <v>261</v>
+      <c r="B40" t="s">
+        <v>260</v>
+      </c>
+      <c r="C40">
+        <v>100</v>
       </c>
       <c r="D40">
-        <v>100</v>
-      </c>
-      <c r="E40">
         <v>39</v>
       </c>
     </row>
-    <row r="41" spans="1:5">
+    <row r="41" spans="1:4">
       <c r="A41">
         <v>40</v>
       </c>
-      <c r="B41">
-        <v>35000</v>
-      </c>
-      <c r="C41" t="s">
-        <v>259</v>
+      <c r="B41" t="s">
+        <v>258</v>
+      </c>
+      <c r="C41">
+        <v>80</v>
       </c>
       <c r="D41">
-        <v>80</v>
-      </c>
-      <c r="E41">
         <v>40</v>
       </c>
     </row>
-    <row r="42" spans="1:5">
+    <row r="42" spans="1:4">
       <c r="A42">
         <v>41</v>
       </c>
-      <c r="B42">
-        <v>6000</v>
-      </c>
-      <c r="C42" t="s">
-        <v>262</v>
+      <c r="B42" t="s">
+        <v>261</v>
+      </c>
+      <c r="C42">
+        <v>250</v>
       </c>
       <c r="D42">
-        <v>250</v>
-      </c>
-      <c r="E42">
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:5">
+    <row r="43" spans="1:4">
       <c r="A43">
         <v>42</v>
       </c>
-      <c r="B43">
-        <v>9000</v>
-      </c>
-      <c r="C43" t="s">
-        <v>262</v>
+      <c r="B43" t="s">
+        <v>261</v>
+      </c>
+      <c r="C43">
+        <v>240</v>
       </c>
       <c r="D43">
-        <v>240</v>
-      </c>
-      <c r="E43">
         <v>42</v>
       </c>
     </row>
-    <row r="44" spans="1:5">
+    <row r="44" spans="1:4">
       <c r="A44">
         <v>43</v>
       </c>
-      <c r="B44">
-        <v>5000</v>
-      </c>
-      <c r="C44" t="s">
-        <v>262</v>
+      <c r="B44" t="s">
+        <v>261</v>
+      </c>
+      <c r="C44">
+        <v>260</v>
       </c>
       <c r="D44">
-        <v>260</v>
-      </c>
-      <c r="E44">
         <v>43</v>
       </c>
     </row>
-    <row r="45" spans="1:5">
+    <row r="45" spans="1:4">
       <c r="A45">
         <v>44</v>
       </c>
-      <c r="B45">
-        <v>10000</v>
-      </c>
-      <c r="C45" t="s">
-        <v>262</v>
+      <c r="B45" t="s">
+        <v>261</v>
+      </c>
+      <c r="C45">
+        <v>180</v>
       </c>
       <c r="D45">
-        <v>180</v>
-      </c>
-      <c r="E45">
         <v>44</v>
       </c>
     </row>
-    <row r="46" spans="1:5">
+    <row r="46" spans="1:4">
       <c r="A46">
         <v>45</v>
       </c>
-      <c r="B46">
-        <v>22000</v>
-      </c>
-      <c r="C46" t="s">
-        <v>261</v>
+      <c r="B46" t="s">
+        <v>260</v>
+      </c>
+      <c r="C46">
+        <v>120</v>
       </c>
       <c r="D46">
-        <v>120</v>
-      </c>
-      <c r="E46">
         <v>45</v>
       </c>
     </row>
-    <row r="47" spans="1:5">
+    <row r="47" spans="1:4">
       <c r="A47">
         <v>46</v>
       </c>
-      <c r="B47">
-        <v>55000</v>
-      </c>
-      <c r="C47" t="s">
-        <v>260</v>
+      <c r="B47" t="s">
+        <v>259</v>
+      </c>
+      <c r="C47">
+        <v>70</v>
       </c>
       <c r="D47">
-        <v>70</v>
-      </c>
-      <c r="E47">
         <v>46</v>
       </c>
     </row>
-    <row r="48" spans="1:5">
+    <row r="48" spans="1:4">
       <c r="A48">
         <v>47</v>
       </c>
-      <c r="B48">
-        <v>18000</v>
-      </c>
-      <c r="C48" t="s">
-        <v>261</v>
+      <c r="B48" t="s">
+        <v>260</v>
+      </c>
+      <c r="C48">
+        <v>90</v>
       </c>
       <c r="D48">
-        <v>90</v>
-      </c>
-      <c r="E48">
         <v>47</v>
       </c>
     </row>
-    <row r="49" spans="1:5">
+    <row r="49" spans="1:4">
       <c r="A49">
         <v>48</v>
       </c>
-      <c r="B49">
-        <v>50000</v>
-      </c>
-      <c r="C49" t="s">
-        <v>259</v>
+      <c r="B49" t="s">
+        <v>258</v>
+      </c>
+      <c r="C49">
+        <v>100</v>
       </c>
       <c r="D49">
-        <v>100</v>
-      </c>
-      <c r="E49">
         <v>48</v>
       </c>
     </row>
-    <row r="50" spans="1:5">
+    <row r="50" spans="1:4">
       <c r="A50">
         <v>49</v>
       </c>
-      <c r="B50">
-        <v>24000</v>
-      </c>
-      <c r="C50" t="s">
-        <v>260</v>
+      <c r="B50" t="s">
+        <v>259</v>
+      </c>
+      <c r="C50">
+        <v>110</v>
       </c>
       <c r="D50">
-        <v>110</v>
-      </c>
-      <c r="E50">
         <v>49</v>
       </c>
     </row>
-    <row r="51" spans="1:5">
+    <row r="51" spans="1:4">
       <c r="A51">
         <v>50</v>
       </c>
-      <c r="B51">
-        <v>10000</v>
-      </c>
-      <c r="C51" t="s">
-        <v>258</v>
+      <c r="B51" t="s">
+        <v>257</v>
+      </c>
+      <c r="C51">
+        <v>210</v>
       </c>
       <c r="D51">
-        <v>210</v>
-      </c>
-      <c r="E51">
         <v>50</v>
       </c>
     </row>
-    <row r="52" spans="1:5">
+    <row r="52" spans="1:4">
       <c r="A52">
         <v>51</v>
       </c>
-      <c r="B52">
-        <v>12000</v>
-      </c>
-      <c r="C52" t="s">
-        <v>260</v>
+      <c r="B52" t="s">
+        <v>259</v>
+      </c>
+      <c r="C52">
+        <v>150</v>
       </c>
       <c r="D52">
-        <v>150</v>
-      </c>
-      <c r="E52">
         <v>51</v>
       </c>
     </row>
-    <row r="53" spans="1:5">
+    <row r="53" spans="1:4">
       <c r="A53">
         <v>52</v>
       </c>
-      <c r="B53">
-        <v>14000</v>
-      </c>
-      <c r="C53" t="s">
-        <v>260</v>
+      <c r="B53" t="s">
+        <v>259</v>
+      </c>
+      <c r="C53">
+        <v>130</v>
       </c>
       <c r="D53">
-        <v>130</v>
-      </c>
-      <c r="E53">
         <v>52</v>
       </c>
     </row>
-    <row r="54" spans="1:5">
+    <row r="54" spans="1:4">
       <c r="A54">
         <v>53</v>
       </c>
-      <c r="B54">
-        <v>9000</v>
-      </c>
-      <c r="C54" t="s">
-        <v>258</v>
+      <c r="B54" t="s">
+        <v>257</v>
+      </c>
+      <c r="C54">
+        <v>200</v>
       </c>
       <c r="D54">
-        <v>200</v>
-      </c>
-      <c r="E54">
         <v>53</v>
       </c>
     </row>
-    <row r="55" spans="1:5">
+    <row r="55" spans="1:4">
       <c r="A55">
         <v>54</v>
       </c>
-      <c r="B55">
-        <v>9000</v>
-      </c>
-      <c r="C55" t="s">
-        <v>258</v>
+      <c r="B55" t="s">
+        <v>257</v>
+      </c>
+      <c r="C55">
+        <v>180</v>
       </c>
       <c r="D55">
-        <v>180</v>
-      </c>
-      <c r="E55">
         <v>54</v>
       </c>
     </row>
-    <row r="56" spans="1:5">
+    <row r="56" spans="1:4">
       <c r="A56">
         <v>55</v>
       </c>
-      <c r="B56">
-        <v>20000</v>
-      </c>
-      <c r="C56" t="s">
-        <v>262</v>
+      <c r="B56" t="s">
+        <v>261</v>
+      </c>
+      <c r="C56">
+        <v>100</v>
       </c>
       <c r="D56">
-        <v>100</v>
-      </c>
-      <c r="E56">
         <v>55</v>
       </c>
     </row>
-    <row r="57" spans="1:5">
+    <row r="57" spans="1:4">
       <c r="A57">
         <v>56</v>
       </c>
-      <c r="B57">
-        <v>12000</v>
-      </c>
-      <c r="C57" t="s">
-        <v>262</v>
+      <c r="B57" t="s">
+        <v>261</v>
+      </c>
+      <c r="C57">
+        <v>120</v>
       </c>
       <c r="D57">
-        <v>120</v>
-      </c>
-      <c r="E57">
         <v>56</v>
       </c>
     </row>
-    <row r="58" spans="1:5">
+    <row r="58" spans="1:4">
       <c r="A58">
         <v>57</v>
       </c>
-      <c r="B58">
-        <v>15000</v>
-      </c>
-      <c r="C58" t="s">
-        <v>262</v>
+      <c r="B58" t="s">
+        <v>261</v>
+      </c>
+      <c r="C58">
+        <v>110</v>
       </c>
       <c r="D58">
-        <v>110</v>
-      </c>
-      <c r="E58">
         <v>57</v>
       </c>
     </row>
-    <row r="59" spans="1:5">
+    <row r="59" spans="1:4">
       <c r="A59">
         <v>58</v>
       </c>
-      <c r="B59">
-        <v>18000</v>
-      </c>
-      <c r="C59" t="s">
-        <v>263</v>
+      <c r="B59" t="s">
+        <v>262</v>
+      </c>
+      <c r="C59">
+        <v>50</v>
       </c>
       <c r="D59">
-        <v>50</v>
-      </c>
-      <c r="E59">
         <v>58</v>
       </c>
     </row>
-    <row r="60" spans="1:5">
+    <row r="60" spans="1:4">
       <c r="A60">
         <v>60</v>
       </c>
-      <c r="B60">
-        <v>35000</v>
-      </c>
-      <c r="C60" t="s">
-        <v>263</v>
+      <c r="B60" t="s">
+        <v>262</v>
+      </c>
+      <c r="C60">
+        <v>35</v>
       </c>
       <c r="D60">
-        <v>35</v>
-      </c>
-      <c r="E60">
         <v>60</v>
       </c>
     </row>
-    <row r="61" spans="1:5">
+    <row r="61" spans="1:4">
       <c r="A61">
         <v>61</v>
       </c>
-      <c r="B61">
-        <v>42000</v>
-      </c>
-      <c r="C61" t="s">
-        <v>259</v>
+      <c r="B61" t="s">
+        <v>258</v>
+      </c>
+      <c r="C61">
+        <v>30</v>
       </c>
       <c r="D61">
-        <v>30</v>
-      </c>
-      <c r="E61">
         <v>61</v>
       </c>
     </row>
-    <row r="62" spans="1:5">
+    <row r="62" spans="1:4">
       <c r="A62">
         <v>62</v>
       </c>
-      <c r="B62">
-        <v>42000</v>
-      </c>
-      <c r="C62" t="s">
-        <v>259</v>
+      <c r="B62" t="s">
+        <v>258</v>
+      </c>
+      <c r="C62">
+        <v>25</v>
       </c>
       <c r="D62">
-        <v>25</v>
-      </c>
-      <c r="E62">
         <v>62</v>
       </c>
     </row>
-    <row r="63" spans="1:5">
+    <row r="63" spans="1:4">
       <c r="A63">
         <v>63</v>
       </c>
-      <c r="B63">
-        <v>28000</v>
-      </c>
-      <c r="C63" t="s">
-        <v>262</v>
+      <c r="B63" t="s">
+        <v>261</v>
+      </c>
+      <c r="C63">
+        <v>60</v>
       </c>
       <c r="D63">
-        <v>60</v>
-      </c>
-      <c r="E63">
         <v>63</v>
       </c>
     </row>
-    <row r="64" spans="1:5">
+    <row r="64" spans="1:4">
       <c r="A64">
         <v>64</v>
       </c>
-      <c r="B64">
-        <v>85000</v>
-      </c>
-      <c r="C64" t="s">
-        <v>261</v>
+      <c r="B64" t="s">
+        <v>260</v>
+      </c>
+      <c r="C64">
+        <v>20</v>
       </c>
       <c r="D64">
-        <v>20</v>
-      </c>
-      <c r="E64">
         <v>64</v>
       </c>
     </row>
-    <row r="65" spans="1:5">
+    <row r="65" spans="1:4">
       <c r="A65">
         <v>65</v>
       </c>
-      <c r="B65">
-        <v>45000</v>
-      </c>
-      <c r="C65" t="s">
-        <v>264</v>
+      <c r="B65" t="s">
+        <v>263</v>
+      </c>
+      <c r="C65">
+        <v>40</v>
       </c>
       <c r="D65">
-        <v>40</v>
-      </c>
-      <c r="E65">
         <v>65</v>
       </c>
     </row>
-    <row r="66" spans="1:5">
+    <row r="66" spans="1:4">
       <c r="A66">
         <v>66</v>
       </c>
-      <c r="B66">
-        <v>45000</v>
-      </c>
-      <c r="C66" t="s">
-        <v>264</v>
+      <c r="B66" t="s">
+        <v>263</v>
+      </c>
+      <c r="C66">
+        <v>40</v>
       </c>
       <c r="D66">
-        <v>40</v>
-      </c>
-      <c r="E66">
         <v>66</v>
       </c>
     </row>
-    <row r="67" spans="1:5">
+    <row r="67" spans="1:4">
       <c r="A67">
         <v>74</v>
       </c>
-      <c r="B67">
-        <v>25000</v>
-      </c>
-      <c r="C67" t="s">
-        <v>263</v>
+      <c r="B67" t="s">
+        <v>262</v>
+      </c>
+      <c r="C67">
+        <v>60</v>
       </c>
       <c r="D67">
-        <v>60</v>
-      </c>
-      <c r="E67">
         <v>74</v>
       </c>
     </row>
-    <row r="68" spans="1:5">
+    <row r="68" spans="1:4">
       <c r="A68">
         <v>75</v>
       </c>
-      <c r="B68">
-        <v>18000</v>
-      </c>
-      <c r="C68" t="s">
-        <v>263</v>
+      <c r="B68" t="s">
+        <v>262</v>
+      </c>
+      <c r="C68">
+        <v>50</v>
       </c>
       <c r="D68">
-        <v>50</v>
-      </c>
-      <c r="E68">
         <v>75</v>
       </c>
     </row>
-    <row r="69" spans="1:5">
+    <row r="69" spans="1:4">
       <c r="A69">
         <v>77</v>
       </c>
-      <c r="B69">
-        <v>22000</v>
-      </c>
-      <c r="C69" t="s">
-        <v>259</v>
+      <c r="B69" t="s">
+        <v>258</v>
+      </c>
+      <c r="C69">
+        <v>90</v>
       </c>
       <c r="D69">
-        <v>90</v>
-      </c>
-      <c r="E69">
         <v>77</v>
       </c>
     </row>
-    <row r="70" spans="1:5">
+    <row r="70" spans="1:4">
       <c r="A70">
         <v>78</v>
       </c>
-      <c r="B70">
-        <v>18000</v>
-      </c>
-      <c r="C70" t="s">
-        <v>265</v>
+      <c r="B70" t="s">
+        <v>264</v>
+      </c>
+      <c r="C70">
+        <v>120</v>
       </c>
       <c r="D70">
-        <v>120</v>
-      </c>
-      <c r="E70">
         <v>78</v>
       </c>
     </row>
-    <row r="71" spans="1:5">
+    <row r="71" spans="1:4">
       <c r="A71">
         <v>79</v>
       </c>
-      <c r="B71">
-        <v>20000</v>
-      </c>
-      <c r="C71" t="s">
-        <v>265</v>
+      <c r="B71" t="s">
+        <v>264</v>
+      </c>
+      <c r="C71">
+        <v>100</v>
       </c>
       <c r="D71">
-        <v>100</v>
-      </c>
-      <c r="E71">
         <v>79</v>
       </c>
     </row>
@@ -6886,6 +6674,797 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00B0444E-33B9-49F0-AC14-74FC5948E165}">
+  <dimension ref="A1:C71"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>265</v>
+      </c>
+      <c r="C1" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>12000</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>13000</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>14000</v>
+      </c>
+      <c r="C4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>10000</v>
+      </c>
+      <c r="C5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>10000</v>
+      </c>
+      <c r="C6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>10000</v>
+      </c>
+      <c r="C7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>12000</v>
+      </c>
+      <c r="C8">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>15000</v>
+      </c>
+      <c r="C9">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>18000</v>
+      </c>
+      <c r="C10">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>18000</v>
+      </c>
+      <c r="C11">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12">
+        <v>35000</v>
+      </c>
+      <c r="C12">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13">
+        <v>28000</v>
+      </c>
+      <c r="C13">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14">
+        <v>45000</v>
+      </c>
+      <c r="C14">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15">
+        <v>5000</v>
+      </c>
+      <c r="C15">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16">
+        <v>8000</v>
+      </c>
+      <c r="C16">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17">
+        <v>4500</v>
+      </c>
+      <c r="C17">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18">
+        <v>9000</v>
+      </c>
+      <c r="C18">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19">
+        <v>22000</v>
+      </c>
+      <c r="C19">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20">
+        <v>22000</v>
+      </c>
+      <c r="C20">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21">
+        <v>55000</v>
+      </c>
+      <c r="C21">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22">
+        <v>20000</v>
+      </c>
+      <c r="C22">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23">
+        <v>45000</v>
+      </c>
+      <c r="C23">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24">
+        <v>22000</v>
+      </c>
+      <c r="C24">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25">
+        <v>10000</v>
+      </c>
+      <c r="C25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26">
+        <v>12000</v>
+      </c>
+      <c r="C26">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27">
+        <v>12000</v>
+      </c>
+      <c r="C27">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28">
+        <v>7000</v>
+      </c>
+      <c r="C28">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29">
+        <v>7000</v>
+      </c>
+      <c r="C29">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30">
+        <v>5000</v>
+      </c>
+      <c r="C30">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31">
+        <v>36000</v>
+      </c>
+      <c r="C31">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32">
+        <v>18000</v>
+      </c>
+      <c r="C32">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33">
+        <v>12000</v>
+      </c>
+      <c r="C33">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34">
+        <v>15000</v>
+      </c>
+      <c r="C34">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35">
+        <v>13000</v>
+      </c>
+      <c r="C35">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36">
+        <v>15000</v>
+      </c>
+      <c r="C36">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37">
+        <v>12000</v>
+      </c>
+      <c r="C37">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38">
+        <v>12000</v>
+      </c>
+      <c r="C38">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3">
+      <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39">
+        <v>16000</v>
+      </c>
+      <c r="C39">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40">
+        <v>18000</v>
+      </c>
+      <c r="C40">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41">
+        <v>35000</v>
+      </c>
+      <c r="C41">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3">
+      <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42">
+        <v>6000</v>
+      </c>
+      <c r="C42">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43">
+        <v>9000</v>
+      </c>
+      <c r="C43">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3">
+      <c r="A44">
+        <v>43</v>
+      </c>
+      <c r="B44">
+        <v>5000</v>
+      </c>
+      <c r="C44">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3">
+      <c r="A45">
+        <v>44</v>
+      </c>
+      <c r="B45">
+        <v>10000</v>
+      </c>
+      <c r="C45">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3">
+      <c r="A46">
+        <v>45</v>
+      </c>
+      <c r="B46">
+        <v>22000</v>
+      </c>
+      <c r="C46">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3">
+      <c r="A47">
+        <v>46</v>
+      </c>
+      <c r="B47">
+        <v>55000</v>
+      </c>
+      <c r="C47">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3">
+      <c r="A48">
+        <v>47</v>
+      </c>
+      <c r="B48">
+        <v>18000</v>
+      </c>
+      <c r="C48">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3">
+      <c r="A49">
+        <v>48</v>
+      </c>
+      <c r="B49">
+        <v>50000</v>
+      </c>
+      <c r="C49">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3">
+      <c r="A50">
+        <v>49</v>
+      </c>
+      <c r="B50">
+        <v>24000</v>
+      </c>
+      <c r="C50">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3">
+      <c r="A51">
+        <v>50</v>
+      </c>
+      <c r="B51">
+        <v>10000</v>
+      </c>
+      <c r="C51">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3">
+      <c r="A52">
+        <v>51</v>
+      </c>
+      <c r="B52">
+        <v>12000</v>
+      </c>
+      <c r="C52">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3">
+      <c r="A53">
+        <v>52</v>
+      </c>
+      <c r="B53">
+        <v>14000</v>
+      </c>
+      <c r="C53">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3">
+      <c r="A54">
+        <v>53</v>
+      </c>
+      <c r="B54">
+        <v>9000</v>
+      </c>
+      <c r="C54">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3">
+      <c r="A55">
+        <v>54</v>
+      </c>
+      <c r="B55">
+        <v>9000</v>
+      </c>
+      <c r="C55">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3">
+      <c r="A56">
+        <v>55</v>
+      </c>
+      <c r="B56">
+        <v>20000</v>
+      </c>
+      <c r="C56">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3">
+      <c r="A57">
+        <v>56</v>
+      </c>
+      <c r="B57">
+        <v>12000</v>
+      </c>
+      <c r="C57">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3">
+      <c r="A58">
+        <v>57</v>
+      </c>
+      <c r="B58">
+        <v>15000</v>
+      </c>
+      <c r="C58">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3">
+      <c r="A59">
+        <v>58</v>
+      </c>
+      <c r="B59">
+        <v>18000</v>
+      </c>
+      <c r="C59">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3">
+      <c r="A60">
+        <v>60</v>
+      </c>
+      <c r="B60">
+        <v>35000</v>
+      </c>
+      <c r="C60">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3">
+      <c r="A61">
+        <v>61</v>
+      </c>
+      <c r="B61">
+        <v>42000</v>
+      </c>
+      <c r="C61">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3">
+      <c r="A62">
+        <v>62</v>
+      </c>
+      <c r="B62">
+        <v>42000</v>
+      </c>
+      <c r="C62">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3">
+      <c r="A63">
+        <v>63</v>
+      </c>
+      <c r="B63">
+        <v>28000</v>
+      </c>
+      <c r="C63">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3">
+      <c r="A64">
+        <v>64</v>
+      </c>
+      <c r="B64">
+        <v>85000</v>
+      </c>
+      <c r="C64">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3">
+      <c r="A65">
+        <v>65</v>
+      </c>
+      <c r="B65">
+        <v>45000</v>
+      </c>
+      <c r="C65">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3">
+      <c r="A66">
+        <v>66</v>
+      </c>
+      <c r="B66">
+        <v>45000</v>
+      </c>
+      <c r="C66">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3">
+      <c r="A67">
+        <v>74</v>
+      </c>
+      <c r="B67">
+        <v>25000</v>
+      </c>
+      <c r="C67">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3">
+      <c r="A68">
+        <v>75</v>
+      </c>
+      <c r="B68">
+        <v>18000</v>
+      </c>
+      <c r="C68">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3">
+      <c r="A69">
+        <v>77</v>
+      </c>
+      <c r="B69">
+        <v>22000</v>
+      </c>
+      <c r="C69">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3">
+      <c r="A70">
+        <v>78</v>
+      </c>
+      <c r="B70">
+        <v>18000</v>
+      </c>
+      <c r="C70">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3">
+      <c r="A71">
+        <v>79</v>
+      </c>
+      <c r="B71">
+        <v>20000</v>
+      </c>
+      <c r="C71">
+        <v>79</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{748F4E0F-BC34-4228-867E-9D0F821705DC}">
   <dimension ref="A1:C42"/>
   <sheetFormatPr defaultRowHeight="15"/>

</xml_diff>

<commit_message>
Refactor Branch and ProductStock models, update mappings
Refactored Branch entity and DTOs to use new fields (Name, Code, contact info, geolocation, status, hours) and removed Country, City, Description. Changed Product to support multiple ProductStocks, linking ProductStock to both Product and Branch. Updated all related specs, mappings, EF configurations, and seeders. Removed Branch validators. Introduced BranchStatus enum and updated Excel seed data. Removed stock status mapping from CartItem and WishlistItem responses.
</commit_message>
<xml_diff>
--- a/src/External/ConvenienceStore.Persistence/Data/ConvenienceStoreData.xlsx
+++ b/src/External/ConvenienceStore.Persistence/Data/ConvenienceStoreData.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30327"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="239" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6A7B0C29-07F3-4D4E-A61B-1D522CD334A4}"/>
+  <xr:revisionPtr revIDLastSave="256" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{09D0E808-62C4-4215-B73B-B4F9F61487A6}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="4" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="5" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Categories" sheetId="1" r:id="rId1"/>
@@ -15,6 +15,7 @@
     <sheet name="ProductStocks" sheetId="4" r:id="rId5"/>
     <sheet name="ProductPrices" sheetId="7" r:id="rId6"/>
     <sheet name="Brands" sheetId="2" r:id="rId7"/>
+    <sheet name="Branchs" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="639" uniqueCount="346">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="676" uniqueCount="378">
   <si>
     <t>Id</t>
   </si>
@@ -839,6 +840,9 @@
     <t>QuantityOnHand</t>
   </si>
   <si>
+    <t>BranchId</t>
+  </si>
+  <si>
     <t>Bottle</t>
   </si>
   <si>
@@ -1104,13 +1108,106 @@
   </si>
   <si>
     <t>Gia công nước giải khát theo yêu cầu khách hàng: nước ép trái cây, nước yến sào cao cấp, nước dừa tươi đóng lon...</t>
+  </si>
+  <si>
+    <t>Code</t>
+  </si>
+  <si>
+    <t>PhoneNumber</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Address</t>
+  </si>
+  <si>
+    <t>Latitude</t>
+  </si>
+  <si>
+    <t>Longitude</t>
+  </si>
+  <si>
+    <t>OpenTime</t>
+  </si>
+  <si>
+    <t>CloseTime</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Thủ Dầu Một</t>
+  </si>
+  <si>
+    <t>BD001</t>
+  </si>
+  <si>
+    <t>bd001@store.local</t>
+  </si>
+  <si>
+    <t>123 Đại lộ Bình Dương, TP. Thủ Dầu Một, Bình Dương</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>Thuận An</t>
+  </si>
+  <si>
+    <t>BD002</t>
+  </si>
+  <si>
+    <t>bd002@store.local</t>
+  </si>
+  <si>
+    <t>45 Nguyễn Văn Tiết, TP. Thuận An, Bình Dương</t>
+  </si>
+  <si>
+    <t>Dĩ An</t>
+  </si>
+  <si>
+    <t>BD003</t>
+  </si>
+  <si>
+    <t>bd003@store.local</t>
+  </si>
+  <si>
+    <t>88 Quốc lộ 1K, TP. Dĩ An, Bình Dương</t>
+  </si>
+  <si>
+    <t>Bến Cát</t>
+  </si>
+  <si>
+    <t>BD004</t>
+  </si>
+  <si>
+    <t>bd004@store.local</t>
+  </si>
+  <si>
+    <t>12 Hùng Vương, TP. Bến Cát, Bình Dương</t>
+  </si>
+  <si>
+    <t>Tân Uyên</t>
+  </si>
+  <si>
+    <t>BD005</t>
+  </si>
+  <si>
+    <t>bd005@store.local</t>
+  </si>
+  <si>
+    <t>99 DT746, TP. Tân Uyên, Bình Dương</t>
+  </si>
+  <si>
+    <t>Inactive</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1134,6 +1231,11 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1156,9 +1258,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="20" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -5668,13 +5772,13 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B485A97C-E092-4E06-B68C-90ECE5645DB1}">
-  <dimension ref="A1:D71"/>
+  <dimension ref="A1:E71"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="3" max="3" width="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -5687,13 +5791,16 @@
       <c r="D1" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="2" spans="1:4">
+      <c r="E1" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C2">
         <v>150</v>
@@ -5701,13 +5808,16 @@
       <c r="D2">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:4">
+      <c r="E2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C3">
         <v>140</v>
@@ -5715,13 +5825,16 @@
       <c r="D3">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:4">
+      <c r="E3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C4">
         <v>120</v>
@@ -5729,13 +5842,16 @@
       <c r="D4">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:4">
+      <c r="E4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C5">
         <v>300</v>
@@ -5743,13 +5859,16 @@
       <c r="D5">
         <v>4</v>
       </c>
-    </row>
-    <row r="6" spans="1:4">
+      <c r="E5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C6">
         <v>250</v>
@@ -5757,13 +5876,16 @@
       <c r="D6">
         <v>5</v>
       </c>
-    </row>
-    <row r="7" spans="1:4">
+      <c r="E6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C7">
         <v>280</v>
@@ -5771,13 +5893,16 @@
       <c r="D7">
         <v>6</v>
       </c>
-    </row>
-    <row r="8" spans="1:4">
+      <c r="E7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C8">
         <v>180</v>
@@ -5785,13 +5910,16 @@
       <c r="D8">
         <v>7</v>
       </c>
-    </row>
-    <row r="9" spans="1:4">
+      <c r="E8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C9">
         <v>160</v>
@@ -5799,13 +5927,16 @@
       <c r="D9">
         <v>8</v>
       </c>
-    </row>
-    <row r="10" spans="1:4">
+      <c r="E9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C10">
         <v>100</v>
@@ -5813,13 +5944,16 @@
       <c r="D10">
         <v>9</v>
       </c>
-    </row>
-    <row r="11" spans="1:4">
+      <c r="E10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C11">
         <v>100</v>
@@ -5827,13 +5961,16 @@
       <c r="D11">
         <v>10</v>
       </c>
-    </row>
-    <row r="12" spans="1:4">
+      <c r="E11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C12">
         <v>80</v>
@@ -5841,13 +5978,16 @@
       <c r="D12">
         <v>11</v>
       </c>
-    </row>
-    <row r="13" spans="1:4">
+      <c r="E12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C13">
         <v>90</v>
@@ -5855,13 +5995,16 @@
       <c r="D13">
         <v>12</v>
       </c>
-    </row>
-    <row r="14" spans="1:4">
+      <c r="E13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
       <c r="A14">
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C14">
         <v>60</v>
@@ -5869,13 +6012,16 @@
       <c r="D14">
         <v>13</v>
       </c>
-    </row>
-    <row r="15" spans="1:4">
+      <c r="E14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C15">
         <v>400</v>
@@ -5883,13 +6029,16 @@
       <c r="D15">
         <v>14</v>
       </c>
-    </row>
-    <row r="16" spans="1:4">
+      <c r="E15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
       <c r="A16">
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C16">
         <v>300</v>
@@ -5897,13 +6046,16 @@
       <c r="D16">
         <v>15</v>
       </c>
-    </row>
-    <row r="17" spans="1:4">
+      <c r="E16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
       <c r="A17">
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C17">
         <v>350</v>
@@ -5911,13 +6063,16 @@
       <c r="D17">
         <v>16</v>
       </c>
-    </row>
-    <row r="18" spans="1:4">
+      <c r="E17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
       <c r="A18">
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C18">
         <v>250</v>
@@ -5925,13 +6080,16 @@
       <c r="D18">
         <v>17</v>
       </c>
-    </row>
-    <row r="19" spans="1:4">
+      <c r="E18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
       <c r="A19">
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C19">
         <v>120</v>
@@ -5939,13 +6097,16 @@
       <c r="D19">
         <v>18</v>
       </c>
-    </row>
-    <row r="20" spans="1:4">
+      <c r="E19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
       <c r="A20">
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C20">
         <v>120</v>
@@ -5953,13 +6114,16 @@
       <c r="D20">
         <v>19</v>
       </c>
-    </row>
-    <row r="21" spans="1:4">
+      <c r="E20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
       <c r="A21">
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C21">
         <v>70</v>
@@ -5967,13 +6131,16 @@
       <c r="D21">
         <v>20</v>
       </c>
-    </row>
-    <row r="22" spans="1:4">
+      <c r="E21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
       <c r="A22">
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C22">
         <v>90</v>
@@ -5981,13 +6148,16 @@
       <c r="D22">
         <v>21</v>
       </c>
-    </row>
-    <row r="23" spans="1:4">
+      <c r="E22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5">
       <c r="A23">
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C23">
         <v>150</v>
@@ -5995,13 +6165,16 @@
       <c r="D23">
         <v>22</v>
       </c>
-    </row>
-    <row r="24" spans="1:4">
+      <c r="E23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5">
       <c r="A24">
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C24">
         <v>120</v>
@@ -6009,13 +6182,16 @@
       <c r="D24">
         <v>23</v>
       </c>
-    </row>
-    <row r="25" spans="1:4">
+      <c r="E24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
       <c r="A25">
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C25">
         <v>220</v>
@@ -6023,13 +6199,16 @@
       <c r="D25">
         <v>24</v>
       </c>
-    </row>
-    <row r="26" spans="1:4">
+      <c r="E25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5">
       <c r="A26">
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C26">
         <v>150</v>
@@ -6037,13 +6216,16 @@
       <c r="D26">
         <v>25</v>
       </c>
-    </row>
-    <row r="27" spans="1:4">
+      <c r="E26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5">
       <c r="A27">
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C27">
         <v>180</v>
@@ -6051,13 +6233,16 @@
       <c r="D27">
         <v>26</v>
       </c>
-    </row>
-    <row r="28" spans="1:4">
+      <c r="E27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5">
       <c r="A28">
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C28">
         <v>500</v>
@@ -6065,13 +6250,16 @@
       <c r="D28">
         <v>27</v>
       </c>
-    </row>
-    <row r="29" spans="1:4">
+      <c r="E28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5">
       <c r="A29">
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C29">
         <v>500</v>
@@ -6079,13 +6267,16 @@
       <c r="D29">
         <v>28</v>
       </c>
-    </row>
-    <row r="30" spans="1:4">
+      <c r="E29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5">
       <c r="A30">
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C30">
         <v>300</v>
@@ -6093,13 +6284,16 @@
       <c r="D30">
         <v>29</v>
       </c>
-    </row>
-    <row r="31" spans="1:4">
+      <c r="E30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5">
       <c r="A31">
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C31">
         <v>80</v>
@@ -6107,13 +6301,16 @@
       <c r="D31">
         <v>30</v>
       </c>
-    </row>
-    <row r="32" spans="1:4">
+      <c r="E31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5">
       <c r="A32">
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C32">
         <v>140</v>
@@ -6121,13 +6318,16 @@
       <c r="D32">
         <v>31</v>
       </c>
-    </row>
-    <row r="33" spans="1:4">
+      <c r="E32">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5">
       <c r="A33">
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C33">
         <v>160</v>
@@ -6135,13 +6335,16 @@
       <c r="D33">
         <v>32</v>
       </c>
-    </row>
-    <row r="34" spans="1:4">
+      <c r="E33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5">
       <c r="A34">
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C34">
         <v>170</v>
@@ -6149,13 +6352,16 @@
       <c r="D34">
         <v>33</v>
       </c>
-    </row>
-    <row r="35" spans="1:4">
+      <c r="E34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5">
       <c r="A35">
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C35">
         <v>120</v>
@@ -6163,13 +6369,16 @@
       <c r="D35">
         <v>34</v>
       </c>
-    </row>
-    <row r="36" spans="1:4">
+      <c r="E35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5">
       <c r="A36">
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C36">
         <v>110</v>
@@ -6177,13 +6386,16 @@
       <c r="D36">
         <v>35</v>
       </c>
-    </row>
-    <row r="37" spans="1:4">
+      <c r="E36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5">
       <c r="A37">
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C37">
         <v>200</v>
@@ -6191,13 +6403,16 @@
       <c r="D37">
         <v>36</v>
       </c>
-    </row>
-    <row r="38" spans="1:4">
+      <c r="E37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5">
       <c r="A38">
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C38">
         <v>180</v>
@@ -6205,13 +6420,16 @@
       <c r="D38">
         <v>37</v>
       </c>
-    </row>
-    <row r="39" spans="1:4">
+      <c r="E38">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5">
       <c r="A39">
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C39">
         <v>120</v>
@@ -6219,13 +6437,16 @@
       <c r="D39">
         <v>38</v>
       </c>
-    </row>
-    <row r="40" spans="1:4">
+      <c r="E39">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5">
       <c r="A40">
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C40">
         <v>100</v>
@@ -6233,13 +6454,16 @@
       <c r="D40">
         <v>39</v>
       </c>
-    </row>
-    <row r="41" spans="1:4">
+      <c r="E40">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5">
       <c r="A41">
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C41">
         <v>80</v>
@@ -6247,13 +6471,16 @@
       <c r="D41">
         <v>40</v>
       </c>
-    </row>
-    <row r="42" spans="1:4">
+      <c r="E41">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5">
       <c r="A42">
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C42">
         <v>250</v>
@@ -6261,13 +6488,16 @@
       <c r="D42">
         <v>41</v>
       </c>
-    </row>
-    <row r="43" spans="1:4">
+      <c r="E42">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5">
       <c r="A43">
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C43">
         <v>240</v>
@@ -6275,13 +6505,16 @@
       <c r="D43">
         <v>42</v>
       </c>
-    </row>
-    <row r="44" spans="1:4">
+      <c r="E43">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5">
       <c r="A44">
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C44">
         <v>260</v>
@@ -6289,13 +6522,16 @@
       <c r="D44">
         <v>43</v>
       </c>
-    </row>
-    <row r="45" spans="1:4">
+      <c r="E44">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5">
       <c r="A45">
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C45">
         <v>180</v>
@@ -6303,13 +6539,16 @@
       <c r="D45">
         <v>44</v>
       </c>
-    </row>
-    <row r="46" spans="1:4">
+      <c r="E45">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5">
       <c r="A46">
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C46">
         <v>120</v>
@@ -6317,13 +6556,16 @@
       <c r="D46">
         <v>45</v>
       </c>
-    </row>
-    <row r="47" spans="1:4">
+      <c r="E46">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5">
       <c r="A47">
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C47">
         <v>70</v>
@@ -6331,13 +6573,16 @@
       <c r="D47">
         <v>46</v>
       </c>
-    </row>
-    <row r="48" spans="1:4">
+      <c r="E47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5">
       <c r="A48">
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C48">
         <v>90</v>
@@ -6345,13 +6590,16 @@
       <c r="D48">
         <v>47</v>
       </c>
-    </row>
-    <row r="49" spans="1:4">
+      <c r="E48">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5">
       <c r="A49">
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C49">
         <v>100</v>
@@ -6359,13 +6607,16 @@
       <c r="D49">
         <v>48</v>
       </c>
-    </row>
-    <row r="50" spans="1:4">
+      <c r="E49">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5">
       <c r="A50">
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C50">
         <v>110</v>
@@ -6373,13 +6624,16 @@
       <c r="D50">
         <v>49</v>
       </c>
-    </row>
-    <row r="51" spans="1:4">
+      <c r="E50">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5">
       <c r="A51">
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C51">
         <v>210</v>
@@ -6387,13 +6641,16 @@
       <c r="D51">
         <v>50</v>
       </c>
-    </row>
-    <row r="52" spans="1:4">
+      <c r="E51">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5">
       <c r="A52">
         <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C52">
         <v>150</v>
@@ -6401,13 +6658,16 @@
       <c r="D52">
         <v>51</v>
       </c>
-    </row>
-    <row r="53" spans="1:4">
+      <c r="E52">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5">
       <c r="A53">
         <v>52</v>
       </c>
       <c r="B53" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C53">
         <v>130</v>
@@ -6415,13 +6675,16 @@
       <c r="D53">
         <v>52</v>
       </c>
-    </row>
-    <row r="54" spans="1:4">
+      <c r="E53">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5">
       <c r="A54">
         <v>53</v>
       </c>
       <c r="B54" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C54">
         <v>200</v>
@@ -6429,13 +6692,16 @@
       <c r="D54">
         <v>53</v>
       </c>
-    </row>
-    <row r="55" spans="1:4">
+      <c r="E54">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5">
       <c r="A55">
         <v>54</v>
       </c>
       <c r="B55" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C55">
         <v>180</v>
@@ -6443,13 +6709,16 @@
       <c r="D55">
         <v>54</v>
       </c>
-    </row>
-    <row r="56" spans="1:4">
+      <c r="E55">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5">
       <c r="A56">
         <v>55</v>
       </c>
       <c r="B56" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C56">
         <v>100</v>
@@ -6457,13 +6726,16 @@
       <c r="D56">
         <v>55</v>
       </c>
-    </row>
-    <row r="57" spans="1:4">
+      <c r="E56">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5">
       <c r="A57">
         <v>56</v>
       </c>
       <c r="B57" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C57">
         <v>120</v>
@@ -6471,13 +6743,16 @@
       <c r="D57">
         <v>56</v>
       </c>
-    </row>
-    <row r="58" spans="1:4">
+      <c r="E57">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5">
       <c r="A58">
         <v>57</v>
       </c>
       <c r="B58" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C58">
         <v>110</v>
@@ -6485,13 +6760,16 @@
       <c r="D58">
         <v>57</v>
       </c>
-    </row>
-    <row r="59" spans="1:4">
+      <c r="E58">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5">
       <c r="A59">
         <v>58</v>
       </c>
       <c r="B59" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C59">
         <v>50</v>
@@ -6499,13 +6777,16 @@
       <c r="D59">
         <v>58</v>
       </c>
-    </row>
-    <row r="60" spans="1:4">
+      <c r="E59">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5">
       <c r="A60">
         <v>60</v>
       </c>
       <c r="B60" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C60">
         <v>35</v>
@@ -6513,13 +6794,16 @@
       <c r="D60">
         <v>60</v>
       </c>
-    </row>
-    <row r="61" spans="1:4">
+      <c r="E60">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5">
       <c r="A61">
         <v>61</v>
       </c>
       <c r="B61" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C61">
         <v>30</v>
@@ -6527,13 +6811,16 @@
       <c r="D61">
         <v>61</v>
       </c>
-    </row>
-    <row r="62" spans="1:4">
+      <c r="E61">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5">
       <c r="A62">
         <v>62</v>
       </c>
       <c r="B62" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C62">
         <v>25</v>
@@ -6541,13 +6828,16 @@
       <c r="D62">
         <v>62</v>
       </c>
-    </row>
-    <row r="63" spans="1:4">
+      <c r="E62">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5">
       <c r="A63">
         <v>63</v>
       </c>
       <c r="B63" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C63">
         <v>60</v>
@@ -6555,13 +6845,16 @@
       <c r="D63">
         <v>63</v>
       </c>
-    </row>
-    <row r="64" spans="1:4">
+      <c r="E63">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5">
       <c r="A64">
         <v>64</v>
       </c>
       <c r="B64" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C64">
         <v>20</v>
@@ -6569,13 +6862,16 @@
       <c r="D64">
         <v>64</v>
       </c>
-    </row>
-    <row r="65" spans="1:4">
+      <c r="E64">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5">
       <c r="A65">
         <v>65</v>
       </c>
       <c r="B65" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C65">
         <v>40</v>
@@ -6583,13 +6879,16 @@
       <c r="D65">
         <v>65</v>
       </c>
-    </row>
-    <row r="66" spans="1:4">
+      <c r="E65">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5">
       <c r="A66">
         <v>66</v>
       </c>
       <c r="B66" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C66">
         <v>40</v>
@@ -6597,13 +6896,16 @@
       <c r="D66">
         <v>66</v>
       </c>
-    </row>
-    <row r="67" spans="1:4">
+      <c r="E66">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5">
       <c r="A67">
         <v>74</v>
       </c>
       <c r="B67" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C67">
         <v>60</v>
@@ -6611,13 +6913,16 @@
       <c r="D67">
         <v>74</v>
       </c>
-    </row>
-    <row r="68" spans="1:4">
+      <c r="E67">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5">
       <c r="A68">
         <v>75</v>
       </c>
       <c r="B68" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C68">
         <v>50</v>
@@ -6625,13 +6930,16 @@
       <c r="D68">
         <v>75</v>
       </c>
-    </row>
-    <row r="69" spans="1:4">
+      <c r="E68">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5">
       <c r="A69">
         <v>77</v>
       </c>
       <c r="B69" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C69">
         <v>90</v>
@@ -6639,13 +6947,16 @@
       <c r="D69">
         <v>77</v>
       </c>
-    </row>
-    <row r="70" spans="1:4">
+      <c r="E69">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5">
       <c r="A70">
         <v>78</v>
       </c>
       <c r="B70" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C70">
         <v>120</v>
@@ -6653,19 +6964,25 @@
       <c r="D70">
         <v>78</v>
       </c>
-    </row>
-    <row r="71" spans="1:4">
+      <c r="E70">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5">
       <c r="A71">
         <v>79</v>
       </c>
       <c r="B71" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C71">
         <v>100</v>
       </c>
       <c r="D71">
         <v>79</v>
+      </c>
+      <c r="E71">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -6683,7 +7000,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C1" t="s">
         <v>194</v>
@@ -7488,10 +7805,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C2" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -7499,10 +7816,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C3" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -7510,10 +7827,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C4" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -7521,10 +7838,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C5" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -7532,10 +7849,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C6" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -7543,10 +7860,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C7" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -7554,10 +7871,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C8" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -7565,10 +7882,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C9" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -7576,10 +7893,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C10" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -7587,10 +7904,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C11" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -7598,10 +7915,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C12" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -7609,10 +7926,10 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C13" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -7620,10 +7937,10 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C14" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -7631,10 +7948,10 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C15" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -7642,10 +7959,10 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C16" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -7653,10 +7970,10 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C17" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -7664,10 +7981,10 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C18" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -7675,10 +7992,10 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C19" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -7686,10 +8003,10 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C20" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -7697,10 +8014,10 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C21" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="22" spans="1:3">
@@ -7708,10 +8025,10 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C22" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -7719,10 +8036,10 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C23" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -7730,10 +8047,10 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C24" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
     </row>
     <row r="25" spans="1:3">
@@ -7741,10 +8058,10 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C25" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
     </row>
     <row r="26" spans="1:3">
@@ -7752,10 +8069,10 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C26" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -7763,10 +8080,10 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C27" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="28" spans="1:3">
@@ -7774,10 +8091,10 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C28" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="29" spans="1:3">
@@ -7785,10 +8102,10 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C29" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -7796,10 +8113,10 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C30" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -7807,10 +8124,10 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="C31" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -7818,10 +8135,10 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C32" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -7829,10 +8146,10 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C33" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="34" spans="1:3">
@@ -7840,10 +8157,10 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C34" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
     </row>
     <row r="35" spans="1:3">
@@ -7851,7 +8168,7 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
     </row>
     <row r="36" spans="1:3">
@@ -7859,10 +8176,10 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="C36" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="37" spans="1:3">
@@ -7870,10 +8187,10 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="C37" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="38" spans="1:3">
@@ -7881,10 +8198,10 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="C38" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
     </row>
     <row r="39" spans="1:3">
@@ -7892,10 +8209,10 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="C39" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
     </row>
     <row r="40" spans="1:3">
@@ -7903,7 +8220,7 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
     </row>
     <row r="41" spans="1:3">
@@ -7911,10 +8228,10 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="C41" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
     </row>
     <row r="42" spans="1:3">
@@ -7922,10 +8239,234 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C42" t="s">
-        <v>345</v>
+        <v>346</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B05EF9F-59D5-4C4B-B6E2-050E3F53E8D0}">
+  <dimension ref="A1:K6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="4" max="4" width="16.5703125" customWidth="1"/>
+    <col min="6" max="6" width="20.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>354</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>357</v>
+      </c>
+      <c r="D2" s="2">
+        <v>2743888888</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>359</v>
+      </c>
+      <c r="G2" s="2">
+        <v>10.980460000000001</v>
+      </c>
+      <c r="H2" s="2">
+        <v>106.651856</v>
+      </c>
+      <c r="I2" s="3">
+        <v>0.25</v>
+      </c>
+      <c r="J2" s="3">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="D3" s="2">
+        <v>2743777777</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="G3" s="2">
+        <v>10.911149999999999</v>
+      </c>
+      <c r="H3" s="2">
+        <v>106.71559000000001</v>
+      </c>
+      <c r="I3" s="3">
+        <v>0.25</v>
+      </c>
+      <c r="J3" s="3">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="D4" s="2">
+        <v>2743666666</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="G4" s="2">
+        <v>10.903890000000001</v>
+      </c>
+      <c r="H4" s="2">
+        <v>106.76945000000001</v>
+      </c>
+      <c r="I4" s="3">
+        <v>0.25</v>
+      </c>
+      <c r="J4" s="3">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="A5" s="2">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="D5" s="2">
+        <v>2743555555</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="G5" s="2">
+        <v>11.1188</v>
+      </c>
+      <c r="H5" s="2">
+        <v>106.6095</v>
+      </c>
+      <c r="I5" s="3">
+        <v>0.25</v>
+      </c>
+      <c r="J5" s="3">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6" s="2">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="D6" s="2">
+        <v>2743444444</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="G6" s="2">
+        <v>11.0525</v>
+      </c>
+      <c r="H6" s="2">
+        <v>106.7569</v>
+      </c>
+      <c r="I6" s="3">
+        <v>0.25</v>
+      </c>
+      <c r="J6" s="3">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>377</v>
       </c>
     </row>
   </sheetData>

</xml_diff>